<commit_message>
Learnt COUNTIF and COUNTIFS
</commit_message>
<xml_diff>
--- a/Excel+LAB+4+Dataset_Dmart_Cleaning_Structuring.xlsx
+++ b/Excel+LAB+4+Dataset_Dmart_Cleaning_Structuring.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Desktop\Advanced Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCC4F610-95FB-4852-9E14-2C3018902338}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F0EF811-5E23-409D-9E87-57D9C06A6768}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,10 +22,13 @@
   <definedNames>
     <definedName name="Category">Dmart_sales_data[Category]</definedName>
     <definedName name="city">Dmart_sales_data[Updated_City]</definedName>
+    <definedName name="customer_type">Dmart_sales_data[customer_type]</definedName>
     <definedName name="discount">Dmart_sales_data[discount]</definedName>
+    <definedName name="order_id">Dmart_sales_data[Column1]</definedName>
     <definedName name="payment_mode">Dmart_sales_data[payment_mode]</definedName>
     <definedName name="Region">Dmart_sales_data[Updated region]</definedName>
     <definedName name="sales">Dmart_sales_data[sales]</definedName>
+    <definedName name="transactions">Dmart_sales_data[payment_mode]</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -47,8 +50,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4620" uniqueCount="632">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4639" uniqueCount="650">
   <si>
     <t>Column1</t>
   </si>
@@ -1944,6 +1969,60 @@
   </si>
   <si>
     <t>Total Sales by Electronics North and more than 40 % discount</t>
+  </si>
+  <si>
+    <t>Data</t>
+  </si>
+  <si>
+    <t>apples</t>
+  </si>
+  <si>
+    <t>oranges</t>
+  </si>
+  <si>
+    <t>peaches</t>
+  </si>
+  <si>
+    <t>Data2</t>
+  </si>
+  <si>
+    <t>Total Orders</t>
+  </si>
+  <si>
+    <t>COUNT</t>
+  </si>
+  <si>
+    <t>COUNTIF</t>
+  </si>
+  <si>
+    <t>Transactions done through Cash</t>
+  </si>
+  <si>
+    <t>Transactions done through Card</t>
+  </si>
+  <si>
+    <t>Transactions done through UPI</t>
+  </si>
+  <si>
+    <t>Find the number of transactions having sales value more than 4000</t>
+  </si>
+  <si>
+    <t>Find the number of transactions having sales value more than 4000 for North Region</t>
+  </si>
+  <si>
+    <t>Find the number of transactions having sales value more than 4000 for East Region</t>
+  </si>
+  <si>
+    <t>Find the number of transactions having sales value more than 4000 for South Region</t>
+  </si>
+  <si>
+    <t>Find the number of transactions having sales value more than 4000 for West Region</t>
+  </si>
+  <si>
+    <t>COUNTIFS</t>
+  </si>
+  <si>
+    <t>Count sales for customer type Member and payment mode is UPI or Card</t>
   </si>
 </sst>
 </file>
@@ -1953,9 +2032,9 @@
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
-    <numFmt numFmtId="167" formatCode="&quot;₹&quot;\ #,##0.00"/>
+    <numFmt numFmtId="166" formatCode="&quot;₹&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2081,8 +2160,21 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12.3"/>
+      <color rgb="FF333333"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF212529"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2113,8 +2205,20 @@
         <bgColor theme="5" tint="0.79998168889431442"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD8D8D8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF4F4F4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="23">
+  <borders count="29">
     <border>
       <left/>
       <right/>
@@ -2345,7 +2449,18 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
         <color indexed="64"/>
       </left>
       <right/>
@@ -2355,11 +2470,74 @@
     </border>
     <border>
       <left/>
-      <right style="thin">
+      <right style="medium">
         <color indexed="64"/>
       </right>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -2367,7 +2545,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="91">
+  <cellXfs count="105">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2517,42 +2695,217 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="18" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="18" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="18" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="18" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="52">
+  <dxfs count="58">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12.3"/>
+        <color rgb="FF333333"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFD8D8D8"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF212529"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF4F4F4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FF212529"/>
+        <name val="Segoe UI"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFF4F4F4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <numFmt numFmtId="3" formatCode="#,##0"/>
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -2614,13 +2967,6 @@
     </dxf>
     <dxf>
       <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
         <left style="thin">
           <color indexed="64"/>
         </left>
@@ -2636,32 +2982,10 @@
       </border>
     </dxf>
     <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
+      <border outline="0">
+        <bottom style="thin">
           <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
+        </bottom>
       </border>
     </dxf>
     <dxf>
@@ -2726,9 +3050,146 @@
     </dxf>
     <dxf>
       <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
       </border>
     </dxf>
     <dxf>
@@ -2742,6 +3203,173 @@
         <top style="thin">
           <color indexed="64"/>
         </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
@@ -3351,281 +3979,6 @@
       </fill>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -3640,28 +3993,28 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D1E78581-CDEC-49EE-B8DC-A227C0757631}" name="Dmart_sales_data" displayName="Dmart_sales_data" ref="A1:Q499" totalsRowShown="0" headerRowDxfId="38" dataDxfId="37" tableBorderDxfId="36">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D1E78581-CDEC-49EE-B8DC-A227C0757631}" name="Dmart_sales_data" displayName="Dmart_sales_data" ref="A1:Q499" totalsRowShown="0" headerRowDxfId="57" dataDxfId="56" tableBorderDxfId="55">
   <autoFilter ref="A1:Q499" xr:uid="{D1E78581-CDEC-49EE-B8DC-A227C0757631}"/>
   <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{8B304A60-B8C9-4979-B67B-B25A9B864B72}" name="Column1" dataDxfId="35"/>
-    <tableColumn id="2" xr3:uid="{2D3F64D4-436B-4836-A733-3255B375685E}" name="Region" dataDxfId="34"/>
-    <tableColumn id="15" xr3:uid="{8F8F9EC8-B524-4266-87C9-B369FF884963}" name="Updated region" dataDxfId="33"/>
-    <tableColumn id="3" xr3:uid="{E344FBA1-63F8-453C-BAB0-8696D5C5ADFA}" name="Category" dataDxfId="32"/>
-    <tableColumn id="4" xr3:uid="{EEDFF6A6-A6B8-4584-81CC-3FEFDA60E218}" name="sales" dataDxfId="31"/>
-    <tableColumn id="17" xr3:uid="{0FE78A95-ABA3-4420-9862-389F567677F4}" name="Sales_Range" dataDxfId="30">
+    <tableColumn id="1" xr3:uid="{8B304A60-B8C9-4979-B67B-B25A9B864B72}" name="Column1" dataDxfId="54"/>
+    <tableColumn id="2" xr3:uid="{2D3F64D4-436B-4836-A733-3255B375685E}" name="Region" dataDxfId="53"/>
+    <tableColumn id="15" xr3:uid="{8F8F9EC8-B524-4266-87C9-B369FF884963}" name="Updated region" dataDxfId="52"/>
+    <tableColumn id="3" xr3:uid="{E344FBA1-63F8-453C-BAB0-8696D5C5ADFA}" name="Category" dataDxfId="51"/>
+    <tableColumn id="4" xr3:uid="{EEDFF6A6-A6B8-4584-81CC-3FEFDA60E218}" name="sales" dataDxfId="50"/>
+    <tableColumn id="17" xr3:uid="{0FE78A95-ABA3-4420-9862-389F567677F4}" name="Sales_Range" dataDxfId="49">
       <calculatedColumnFormula>IF(Dmart_sales_data[[#This Row],[sales]]&gt;3000,"High Sales",IF(Dmart_sales_data[[#This Row],[sales]]&gt;1000,"Medium Sales","Low Sales"))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{B480F4CD-1259-4AB9-84E7-ADE183D66042}" name="discount" dataDxfId="29"/>
-    <tableColumn id="6" xr3:uid="{031D638C-25E8-4D1B-BC09-4AA98712CA5F}" name="quantity" dataDxfId="28"/>
-    <tableColumn id="7" xr3:uid="{6F6EB0D8-424B-4AC8-81C9-7C00315E2B39}" name="order_date" dataDxfId="27"/>
-    <tableColumn id="8" xr3:uid="{0655DCF6-A9AE-4DBC-8BCD-0DDB91A76E3F}" name="delivery_date" dataDxfId="26"/>
-    <tableColumn id="9" xr3:uid="{4A08809E-03F7-4D5D-91CC-E0D9BC4E6CCD}" name="customer_type" dataDxfId="25"/>
-    <tableColumn id="10" xr3:uid="{1B22ACAF-6F45-4EF9-BD4D-3882847DEADD}" name="customer_type2" dataDxfId="24"/>
-    <tableColumn id="11" xr3:uid="{1AAA8999-D7A1-4DB5-B4DA-131DA9CFBC1D}" name="payment_mode" dataDxfId="23"/>
-    <tableColumn id="12" xr3:uid="{47AC25B1-7621-493D-B41B-C4A660573B07}" name="profit" dataDxfId="22"/>
-    <tableColumn id="14" xr3:uid="{285DAA76-019F-4DAE-9C58-731537A4E5A8}" name="Updated_City" dataDxfId="21"/>
-    <tableColumn id="13" xr3:uid="{B1583274-EA92-4587-97FE-7E9FCE51D726}" name="city" dataDxfId="20"/>
-    <tableColumn id="18" xr3:uid="{740C088C-8609-4AAD-81B8-DF0D9B02079A}" name="Discount or Not" dataDxfId="19">
+    <tableColumn id="5" xr3:uid="{B480F4CD-1259-4AB9-84E7-ADE183D66042}" name="discount" dataDxfId="48"/>
+    <tableColumn id="6" xr3:uid="{031D638C-25E8-4D1B-BC09-4AA98712CA5F}" name="quantity" dataDxfId="47"/>
+    <tableColumn id="7" xr3:uid="{6F6EB0D8-424B-4AC8-81C9-7C00315E2B39}" name="order_date" dataDxfId="46"/>
+    <tableColumn id="8" xr3:uid="{0655DCF6-A9AE-4DBC-8BCD-0DDB91A76E3F}" name="delivery_date" dataDxfId="45"/>
+    <tableColumn id="9" xr3:uid="{4A08809E-03F7-4D5D-91CC-E0D9BC4E6CCD}" name="customer_type" dataDxfId="44"/>
+    <tableColumn id="10" xr3:uid="{1B22ACAF-6F45-4EF9-BD4D-3882847DEADD}" name="customer_type2" dataDxfId="43"/>
+    <tableColumn id="11" xr3:uid="{1AAA8999-D7A1-4DB5-B4DA-131DA9CFBC1D}" name="payment_mode" dataDxfId="42"/>
+    <tableColumn id="12" xr3:uid="{47AC25B1-7621-493D-B41B-C4A660573B07}" name="profit" dataDxfId="41"/>
+    <tableColumn id="14" xr3:uid="{285DAA76-019F-4DAE-9C58-731537A4E5A8}" name="Updated_City" dataDxfId="40"/>
+    <tableColumn id="13" xr3:uid="{B1583274-EA92-4587-97FE-7E9FCE51D726}" name="city" dataDxfId="39"/>
+    <tableColumn id="18" xr3:uid="{740C088C-8609-4AAD-81B8-DF0D9B02079A}" name="Discount or Not" dataDxfId="38">
       <calculatedColumnFormula>IF(AND(Dmart_sales_data[[#This Row],[customer_type2]]="Member",OR(Dmart_sales_data[[#This Row],[payment_mode]]="UPI",Dmart_sales_data[[#This Row],[payment_mode]]="Card")),"yes","No")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3670,7 +4023,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{0A6E07FC-F19B-467B-A96D-152F49BC9C39}" name="Table3" displayName="Table3" ref="A1:G5" totalsRowShown="0" headerRowDxfId="18" tableBorderDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{0A6E07FC-F19B-467B-A96D-152F49BC9C39}" name="Table3" displayName="Table3" ref="A1:G5" totalsRowShown="0" headerRowDxfId="37" tableBorderDxfId="36">
   <autoFilter ref="A1:G5" xr:uid="{0A6E07FC-F19B-467B-A96D-152F49BC9C39}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{C83CD628-8037-4113-B34D-19B4409139C8}" name="First_Name"/>
@@ -3686,7 +4039,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{591FFA04-0D55-47FF-B03F-46AEB7B93CCC}" name="Table1" displayName="Table1" ref="E7:M11" totalsRowShown="0" headerRowDxfId="16" headerRowBorderDxfId="15" tableBorderDxfId="14" totalsRowBorderDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{591FFA04-0D55-47FF-B03F-46AEB7B93CCC}" name="Table1" displayName="Table1" ref="E7:M11" totalsRowShown="0" headerRowDxfId="35" headerRowBorderDxfId="34" tableBorderDxfId="33" totalsRowBorderDxfId="32">
   <autoFilter ref="E7:M11" xr:uid="{591FFA04-0D55-47FF-B03F-46AEB7B93CCC}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{7A511605-F386-44F8-8EA9-21F82B34DE6B}" name="First_Name"/>
@@ -3704,24 +4057,24 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{C4582CC2-34E1-4108-B90B-B0A79AC476DF}" name="Table4" displayName="Table4" ref="H18:J23" totalsRowShown="0" headerRowBorderDxfId="51" tableBorderDxfId="50" totalsRowBorderDxfId="49">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{C4582CC2-34E1-4108-B90B-B0A79AC476DF}" name="Table4" displayName="Table4" ref="H18:J23" totalsRowShown="0" headerRowBorderDxfId="31" tableBorderDxfId="30" totalsRowBorderDxfId="29">
   <autoFilter ref="H18:J23" xr:uid="{C4582CC2-34E1-4108-B90B-B0A79AC476DF}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{2E1B0446-2B2E-4C3D-A1EE-391AF9212486}" name="Name " dataDxfId="48"/>
-    <tableColumn id="2" xr3:uid="{19AB838D-F57F-4448-AE00-5E4AA9FB304C}" name="Salary" dataDxfId="47"/>
-    <tableColumn id="3" xr3:uid="{B096BCFB-275E-45AA-A72E-D0C36078B65E}" name="Bonus" dataDxfId="46"/>
+    <tableColumn id="1" xr3:uid="{2E1B0446-2B2E-4C3D-A1EE-391AF9212486}" name="Name " dataDxfId="28"/>
+    <tableColumn id="2" xr3:uid="{19AB838D-F57F-4448-AE00-5E4AA9FB304C}" name="Salary" dataDxfId="27"/>
+    <tableColumn id="3" xr3:uid="{B096BCFB-275E-45AA-A72E-D0C36078B65E}" name="Bonus" dataDxfId="26"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{EDE8ED26-A613-4F4E-A465-CC70B9528A2A}" name="Table5" displayName="Table5" ref="H8:J13" totalsRowShown="0" headerRowDxfId="45" headerRowBorderDxfId="44" tableBorderDxfId="43" totalsRowBorderDxfId="42">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{EDE8ED26-A613-4F4E-A465-CC70B9528A2A}" name="Table5" displayName="Table5" ref="H8:J13" totalsRowShown="0" headerRowDxfId="25" headerRowBorderDxfId="24" tableBorderDxfId="23" totalsRowBorderDxfId="22">
   <autoFilter ref="H8:J13" xr:uid="{EDE8ED26-A613-4F4E-A465-CC70B9528A2A}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{CFB5A7CD-331C-4C43-96A8-0EF34910777D}" name="Name " dataDxfId="41"/>
-    <tableColumn id="2" xr3:uid="{CB401229-AA4D-4F02-997A-EECEC42124A1}" name="Marks" dataDxfId="40"/>
-    <tableColumn id="3" xr3:uid="{032BA486-4C96-46E4-9FCC-835E6841B1B4}" name="Grade" dataDxfId="39">
+    <tableColumn id="1" xr3:uid="{CFB5A7CD-331C-4C43-96A8-0EF34910777D}" name="Name " dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{CB401229-AA4D-4F02-997A-EECEC42124A1}" name="Marks" dataDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{032BA486-4C96-46E4-9FCC-835E6841B1B4}" name="Grade" dataDxfId="19">
       <calculatedColumnFormula>IF(I9&gt;=90,"A++",IF(I9&gt;75,"A+",IF(I9&gt;60,"A",IF(I9&gt;40,"B","Fail"))))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3730,12 +4083,12 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{1A0C1234-3244-41FE-AADF-1A185E3361D9}" name="Table6" displayName="Table6" ref="P17:R22" totalsRowShown="0" headerRowDxfId="6" headerRowBorderDxfId="11" tableBorderDxfId="12" totalsRowBorderDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{1A0C1234-3244-41FE-AADF-1A185E3361D9}" name="Table6" displayName="Table6" ref="P17:R22" totalsRowShown="0" headerRowDxfId="18" headerRowBorderDxfId="17" tableBorderDxfId="16" totalsRowBorderDxfId="15">
   <autoFilter ref="P17:R22" xr:uid="{1A0C1234-3244-41FE-AADF-1A185E3361D9}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{B127EBF8-5637-44F7-83D3-381997DBE027}" name="Number 1" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{C43106B6-1733-443D-94FA-BECDAC1C755A}" name="Number 2" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{F76B590F-EE8E-45BA-9CE4-30BC585483D7}" name="Division" dataDxfId="7">
+    <tableColumn id="1" xr3:uid="{B127EBF8-5637-44F7-83D3-381997DBE027}" name="Number 1" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{C43106B6-1733-443D-94FA-BECDAC1C755A}" name="Number 2" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{F76B590F-EE8E-45BA-9CE4-30BC585483D7}" name="Division" dataDxfId="12">
       <calculatedColumnFormula>IFERROR(P18/Q18,"Cannot Devide by Zero")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3744,14 +4097,25 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{DACE1BBE-C5AD-43B2-961F-3CA9A2EB2A9F}" name="Table8" displayName="Table8" ref="B3:D9" totalsRowShown="0" headerRowBorderDxfId="4" tableBorderDxfId="5" totalsRowBorderDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{DACE1BBE-C5AD-43B2-961F-3CA9A2EB2A9F}" name="Table8" displayName="Table8" ref="B3:D9" totalsRowShown="0" headerRowBorderDxfId="11" tableBorderDxfId="10" totalsRowBorderDxfId="9">
   <autoFilter ref="B3:D9" xr:uid="{DACE1BBE-C5AD-43B2-961F-3CA9A2EB2A9F}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{01EE2967-652D-4F72-8D82-47940A310F22}" name="Category" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{83D94CD6-8657-4942-BDBA-E7199934938C}" name="Food" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{84FFB931-E43C-401F-A346-99CA6CFFFDBA}" name="Sales" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{01EE2967-652D-4F72-8D82-47940A310F22}" name="Category" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{83D94CD6-8657-4942-BDBA-E7199934938C}" name="Food" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{84FFB931-E43C-401F-A346-99CA6CFFFDBA}" name="Sales" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight18" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{D282ED5D-22A6-415A-A10A-2B4A8091F761}" name="Table7" displayName="Table7" ref="B16:C20" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="4" tableBorderDxfId="5" totalsRowBorderDxfId="3">
+  <autoFilter ref="B16:C20" xr:uid="{D282ED5D-22A6-415A-A10A-2B4A8091F761}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{0063F624-5548-4FC5-A9F7-B87EB616BE8D}" name="Data" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{ACA1AE24-A257-4956-B7F8-372ACF52726B}" name="Data2" dataDxfId="1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -3973,7 +4337,7 @@
     <col min="16" max="16" width="15" customWidth="1"/>
     <col min="17" max="17" width="23.21875" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="8.6640625" customWidth="1"/>
-    <col min="19" max="19" width="50.77734375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="68.88671875" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="15.88671875" customWidth="1"/>
     <col min="21" max="26" width="8.6640625" customWidth="1"/>
   </cols>
@@ -4174,7 +4538,7 @@
       <c r="AA3" s="1"/>
       <c r="AB3" s="1"/>
     </row>
-    <row r="4" spans="1:28" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="13" t="s">
         <v>23</v>
       </c>
@@ -4240,7 +4604,7 @@
       <c r="AA4" s="1"/>
       <c r="AB4" s="1"/>
     </row>
-    <row r="5" spans="1:28" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
         <v>28</v>
       </c>
@@ -4295,10 +4659,10 @@
         <v>yes</v>
       </c>
       <c r="R5" s="1"/>
-      <c r="S5" s="81" t="s">
+      <c r="S5" s="80" t="s">
         <v>629</v>
       </c>
-      <c r="T5" s="82"/>
+      <c r="T5" s="87"/>
       <c r="U5" s="1"/>
       <c r="V5" s="1"/>
       <c r="W5" s="1"/>
@@ -4363,10 +4727,10 @@
         <v>No</v>
       </c>
       <c r="R6" s="1"/>
-      <c r="S6" s="83" t="s">
+      <c r="S6" s="88" t="s">
         <v>613</v>
       </c>
-      <c r="T6" s="84">
+      <c r="T6" s="95">
         <f>SUMIF(Dmart_sales_data[payment_mode],"=UPI",Dmart_sales_data[sales])</f>
         <v>386412.25</v>
       </c>
@@ -4434,8 +4798,8 @@
         <v>yes</v>
       </c>
       <c r="R7" s="1"/>
-      <c r="S7" s="85"/>
-      <c r="T7" s="84"/>
+      <c r="S7" s="96"/>
+      <c r="T7" s="95"/>
       <c r="U7" s="1"/>
       <c r="V7" s="1"/>
       <c r="W7" s="1"/>
@@ -4500,10 +4864,10 @@
         <v>No</v>
       </c>
       <c r="R8" s="1"/>
-      <c r="S8" s="83" t="s">
+      <c r="S8" s="88" t="s">
         <v>614</v>
       </c>
-      <c r="T8" s="84">
+      <c r="T8" s="95">
         <f>SUMIF(Dmart_sales_data[payment_mode],"=Cash",Dmart_sales_data[sales])</f>
         <v>522964.3</v>
       </c>
@@ -4571,8 +4935,8 @@
         <v>No</v>
       </c>
       <c r="R9" s="1"/>
-      <c r="S9" s="85"/>
-      <c r="T9" s="84"/>
+      <c r="S9" s="96"/>
+      <c r="T9" s="95"/>
       <c r="U9" s="1"/>
       <c r="V9" s="1"/>
       <c r="W9" s="1"/>
@@ -4582,7 +4946,7 @@
       <c r="AA9" s="1"/>
       <c r="AB9" s="1"/>
     </row>
-    <row r="10" spans="1:28" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="13" t="s">
         <v>40</v>
       </c>
@@ -4637,10 +5001,10 @@
         <v>No</v>
       </c>
       <c r="R10" s="1"/>
-      <c r="S10" s="86" t="s">
+      <c r="S10" s="90" t="s">
         <v>615</v>
       </c>
-      <c r="T10" s="87">
+      <c r="T10" s="99">
         <f>SUMIF(Dmart_sales_data[payment_mode],"=Card",Dmart_sales_data[sales])</f>
         <v>413292.63999999996</v>
       </c>
@@ -4653,7 +5017,7 @@
       <c r="AA10" s="1"/>
       <c r="AB10" s="1"/>
     </row>
-    <row r="11" spans="1:28" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="8" t="s">
         <v>42</v>
       </c>
@@ -4719,7 +5083,7 @@
       <c r="AA11" s="1"/>
       <c r="AB11" s="1"/>
     </row>
-    <row r="12" spans="1:28" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:28" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="13" t="s">
         <v>43</v>
       </c>
@@ -4774,10 +5138,10 @@
         <v>No</v>
       </c>
       <c r="R12" s="1"/>
-      <c r="S12" s="81" t="s">
+      <c r="S12" s="80" t="s">
         <v>630</v>
       </c>
-      <c r="T12" s="82"/>
+      <c r="T12" s="87"/>
       <c r="U12" s="1"/>
       <c r="V12" s="1"/>
       <c r="W12" s="1"/>
@@ -4842,10 +5206,10 @@
         <v>No</v>
       </c>
       <c r="R13" s="1"/>
-      <c r="S13" s="83" t="s">
+      <c r="S13" s="88" t="s">
         <v>628</v>
       </c>
-      <c r="T13" s="84">
+      <c r="T13" s="95">
         <f>SUMIFS(Dmart_sales_data[sales],Dmart_sales_data[Category],"=Clothing",Dmart_sales_data[Updated region],"=East")</f>
         <v>60655.859999999993</v>
       </c>
@@ -4913,8 +5277,8 @@
         <v>No</v>
       </c>
       <c r="R14" s="1"/>
-      <c r="S14" s="85"/>
-      <c r="T14" s="88"/>
+      <c r="S14" s="96"/>
+      <c r="T14" s="89"/>
       <c r="U14" s="1"/>
       <c r="V14" s="1"/>
       <c r="W14" s="1"/>
@@ -4924,7 +5288,7 @@
       <c r="AA14" s="1"/>
       <c r="AB14" s="1"/>
     </row>
-    <row r="15" spans="1:28" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:28" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="8" t="s">
         <v>47</v>
       </c>
@@ -4979,10 +5343,10 @@
         <v>No</v>
       </c>
       <c r="R15" s="1"/>
-      <c r="S15" s="89" t="s">
+      <c r="S15" s="97" t="s">
         <v>631</v>
       </c>
-      <c r="T15" s="90">
+      <c r="T15" s="98">
         <f>SUMIFS(Dmart_sales_data[sales],Dmart_sales_data[Category],"Electronics",Dmart_sales_data[Updated region],"North",Dmart_sales_data[discount],"&gt;0.40")</f>
         <v>36091.269999999997</v>
       </c>
@@ -5061,7 +5425,7 @@
       <c r="AA16" s="1"/>
       <c r="AB16" s="1"/>
     </row>
-    <row r="17" spans="1:28" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:28" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="8" t="s">
         <v>50</v>
       </c>
@@ -5127,7 +5491,7 @@
       <c r="AA17" s="1"/>
       <c r="AB17" s="1"/>
     </row>
-    <row r="18" spans="1:28" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:28" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="13" t="s">
         <v>51</v>
       </c>
@@ -5182,8 +5546,10 @@
         <v>yes</v>
       </c>
       <c r="R18" s="1"/>
-      <c r="S18" s="1"/>
-      <c r="T18" s="19"/>
+      <c r="S18" s="92" t="s">
+        <v>638</v>
+      </c>
+      <c r="T18" s="93"/>
       <c r="U18" s="19"/>
       <c r="V18" s="1"/>
       <c r="W18" s="1"/>
@@ -5193,7 +5559,7 @@
       <c r="AA18" s="1"/>
       <c r="AB18" s="1"/>
     </row>
-    <row r="19" spans="1:28" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:28" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="8" t="s">
         <v>53</v>
       </c>
@@ -5248,8 +5614,13 @@
         <v>No</v>
       </c>
       <c r="R19" s="1"/>
-      <c r="S19" s="1"/>
-      <c r="T19" s="1"/>
+      <c r="S19" s="94" t="s">
+        <v>637</v>
+      </c>
+      <c r="T19" s="91">
+        <f>COUNT(sales)</f>
+        <v>498</v>
+      </c>
       <c r="U19" s="1"/>
       <c r="V19" s="1"/>
       <c r="W19" s="1"/>
@@ -5259,7 +5630,7 @@
       <c r="AA19" s="1"/>
       <c r="AB19" s="1"/>
     </row>
-    <row r="20" spans="1:28" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:28" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="13" t="s">
         <v>54</v>
       </c>
@@ -5325,7 +5696,7 @@
       <c r="AA20" s="1"/>
       <c r="AB20" s="1"/>
     </row>
-    <row r="21" spans="1:28" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:28" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="8" t="s">
         <v>56</v>
       </c>
@@ -5380,8 +5751,10 @@
         <v>No</v>
       </c>
       <c r="R21" s="1"/>
-      <c r="S21" s="1"/>
-      <c r="T21" s="1"/>
+      <c r="S21" s="92" t="s">
+        <v>639</v>
+      </c>
+      <c r="T21" s="87"/>
       <c r="U21" s="1"/>
       <c r="V21" s="1"/>
       <c r="W21" s="1"/>
@@ -5446,8 +5819,13 @@
         <v>No</v>
       </c>
       <c r="R22" s="1"/>
-      <c r="S22" s="1"/>
-      <c r="T22" s="1"/>
+      <c r="S22" s="88" t="s">
+        <v>640</v>
+      </c>
+      <c r="T22" s="89" cm="1">
+        <f t="array" ref="T22">COUNTIF(transactions,"Cash")</f>
+        <v>185</v>
+      </c>
       <c r="U22" s="1"/>
       <c r="V22" s="1"/>
       <c r="W22" s="1"/>
@@ -5512,8 +5890,13 @@
         <v>No</v>
       </c>
       <c r="R23" s="1"/>
-      <c r="S23" s="1"/>
-      <c r="T23" s="1"/>
+      <c r="S23" s="88" t="s">
+        <v>641</v>
+      </c>
+      <c r="T23" s="89" cm="1">
+        <f t="array" ref="T23">COUNTIF(transactions,"Card")</f>
+        <v>164</v>
+      </c>
       <c r="U23" s="1"/>
       <c r="V23" s="1"/>
       <c r="W23" s="1"/>
@@ -5523,7 +5906,7 @@
       <c r="AA23" s="1"/>
       <c r="AB23" s="1"/>
     </row>
-    <row r="24" spans="1:28" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:28" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="13" t="s">
         <v>60</v>
       </c>
@@ -5578,8 +5961,13 @@
         <v>No</v>
       </c>
       <c r="R24" s="1"/>
-      <c r="S24" s="1"/>
-      <c r="T24" s="1"/>
+      <c r="S24" s="90" t="s">
+        <v>642</v>
+      </c>
+      <c r="T24" s="91" cm="1">
+        <f t="array" ref="T24">COUNTIF(transactions,"UPI")</f>
+        <v>149</v>
+      </c>
       <c r="U24" s="1"/>
       <c r="V24" s="1"/>
       <c r="W24" s="1"/>
@@ -5589,7 +5977,7 @@
       <c r="AA24" s="1"/>
       <c r="AB24" s="1"/>
     </row>
-    <row r="25" spans="1:28" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:28" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="8" t="s">
         <v>61</v>
       </c>
@@ -5644,8 +6032,13 @@
         <v>No</v>
       </c>
       <c r="R25" s="1"/>
-      <c r="S25" s="1"/>
-      <c r="T25" s="1"/>
+      <c r="S25" s="103" t="s">
+        <v>643</v>
+      </c>
+      <c r="T25" s="104" cm="1">
+        <f t="array" ref="T25">COUNTIF(sales,"&gt;4000")</f>
+        <v>115</v>
+      </c>
       <c r="U25" s="1"/>
       <c r="V25" s="1"/>
       <c r="W25" s="1"/>
@@ -5776,8 +6169,6 @@
         <v>No</v>
       </c>
       <c r="R27" s="1"/>
-      <c r="S27" s="1"/>
-      <c r="T27" s="1"/>
       <c r="U27" s="1"/>
       <c r="V27" s="1"/>
       <c r="W27" s="1"/>
@@ -5787,7 +6178,7 @@
       <c r="AA27" s="1"/>
       <c r="AB27" s="1"/>
     </row>
-    <row r="28" spans="1:28" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:28" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="13" t="s">
         <v>66</v>
       </c>
@@ -5853,7 +6244,7 @@
       <c r="AA28" s="1"/>
       <c r="AB28" s="1"/>
     </row>
-    <row r="29" spans="1:28" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:28" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="8" t="s">
         <v>67</v>
       </c>
@@ -5908,8 +6299,10 @@
         <v>No</v>
       </c>
       <c r="R29" s="1"/>
-      <c r="S29" s="1"/>
-      <c r="T29" s="1"/>
+      <c r="S29" s="80" t="s">
+        <v>648</v>
+      </c>
+      <c r="T29" s="87"/>
       <c r="U29" s="1"/>
       <c r="V29" s="1"/>
       <c r="W29" s="1"/>
@@ -5974,8 +6367,13 @@
         <v>yes</v>
       </c>
       <c r="R30" s="1"/>
-      <c r="S30" s="1"/>
-      <c r="T30" s="1"/>
+      <c r="S30" s="101" t="s">
+        <v>644</v>
+      </c>
+      <c r="T30" s="89" cm="1">
+        <f t="array" ref="T30">COUNTIFS(sales,"&gt;4000",Region,"North")</f>
+        <v>32</v>
+      </c>
       <c r="U30" s="1"/>
       <c r="V30" s="1"/>
       <c r="W30" s="1"/>
@@ -6040,8 +6438,13 @@
         <v>No</v>
       </c>
       <c r="R31" s="1"/>
-      <c r="S31" s="1"/>
-      <c r="T31" s="1"/>
+      <c r="S31" s="101" t="s">
+        <v>645</v>
+      </c>
+      <c r="T31" s="89" cm="1">
+        <f t="array" ref="T31">COUNTIFS(sales,"&gt;4000",Region,"East")</f>
+        <v>29</v>
+      </c>
       <c r="U31" s="1"/>
       <c r="V31" s="1"/>
       <c r="W31" s="1"/>
@@ -6106,8 +6509,13 @@
         <v>No</v>
       </c>
       <c r="R32" s="1"/>
-      <c r="S32" s="1"/>
-      <c r="T32" s="1"/>
+      <c r="S32" s="101" t="s">
+        <v>646</v>
+      </c>
+      <c r="T32" s="89" cm="1">
+        <f t="array" ref="T32">COUNTIFS(sales,"&gt;4000",Region,"South")</f>
+        <v>27</v>
+      </c>
       <c r="U32" s="1"/>
       <c r="V32" s="1"/>
       <c r="W32" s="1"/>
@@ -6117,7 +6525,7 @@
       <c r="AA32" s="1"/>
       <c r="AB32" s="1"/>
     </row>
-    <row r="33" spans="1:28" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:28" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A33" s="8" t="s">
         <v>72</v>
       </c>
@@ -6172,8 +6580,13 @@
         <v>No</v>
       </c>
       <c r="R33" s="1"/>
-      <c r="S33" s="1"/>
-      <c r="T33" s="1"/>
+      <c r="S33" s="102" t="s">
+        <v>647</v>
+      </c>
+      <c r="T33" s="91" cm="1">
+        <f t="array" ref="T33">COUNTIFS(sales,"&gt;4000",Region,"West")</f>
+        <v>27</v>
+      </c>
       <c r="U33" s="1"/>
       <c r="V33" s="1"/>
       <c r="W33" s="1"/>
@@ -6370,8 +6783,13 @@
         <v>No</v>
       </c>
       <c r="R36" s="1"/>
-      <c r="S36" s="1"/>
-      <c r="T36" s="1"/>
+      <c r="S36" s="100" t="s">
+        <v>649</v>
+      </c>
+      <c r="T36" s="1" cm="1">
+        <f t="array" ref="T36">SUM(COUNTIFS(customer_type,"Member",payment_mode,{"Card","UPI"}))</f>
+        <v>97</v>
+      </c>
       <c r="U36" s="1"/>
       <c r="V36" s="1"/>
       <c r="W36" s="1"/>
@@ -51590,11 +52008,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEF34D78-29E1-4CCD-BF36-EC79D09F917E}">
-  <dimension ref="B3:G9"/>
+  <dimension ref="B3:G20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.88671875" style="75"/>
     <col min="6" max="6" width="23.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -51605,7 +52022,7 @@
       <c r="C3" s="73" t="s">
         <v>616</v>
       </c>
-      <c r="D3" s="79" t="s">
+      <c r="D3" s="78" t="s">
         <v>617</v>
       </c>
     </row>
@@ -51616,7 +52033,7 @@
       <c r="C4" s="71" t="s">
         <v>619</v>
       </c>
-      <c r="D4" s="76">
+      <c r="D4" s="75">
         <v>2300</v>
       </c>
     </row>
@@ -51627,7 +52044,7 @@
       <c r="C5" s="71" t="s">
         <v>620</v>
       </c>
-      <c r="D5" s="77">
+      <c r="D5" s="76">
         <v>5500</v>
       </c>
     </row>
@@ -51638,7 +52055,7 @@
       <c r="C6" s="71" t="s">
         <v>622</v>
       </c>
-      <c r="D6" s="78">
+      <c r="D6" s="77">
         <v>800</v>
       </c>
       <c r="F6" s="70" t="s">
@@ -51654,7 +52071,7 @@
       <c r="C7" s="71" t="s">
         <v>623</v>
       </c>
-      <c r="D7" s="78">
+      <c r="D7" s="77">
         <v>400</v>
       </c>
     </row>
@@ -51665,7 +52082,7 @@
       <c r="C8" s="71" t="s">
         <v>624</v>
       </c>
-      <c r="D8" s="77">
+      <c r="D8" s="76">
         <v>4200</v>
       </c>
       <c r="F8" s="70" t="s">
@@ -51683,14 +52100,59 @@
       <c r="C9" s="74" t="s">
         <v>625</v>
       </c>
-      <c r="D9" s="80">
+      <c r="D9" s="79">
         <v>1200</v>
+      </c>
+    </row>
+    <row r="16" spans="2:7" ht="20.399999999999999" x14ac:dyDescent="0.3">
+      <c r="B16" s="83" t="s">
+        <v>632</v>
+      </c>
+      <c r="C16" s="84" t="s">
+        <v>636</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="B17" s="81" t="s">
+        <v>633</v>
+      </c>
+      <c r="C17" s="82">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="B18" s="81" t="s">
+        <v>634</v>
+      </c>
+      <c r="C18" s="82">
+        <v>54</v>
+      </c>
+      <c r="E18">
+        <f>COUNTIF(B17:B20,"oranges")</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="2:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="B19" s="81" t="s">
+        <v>635</v>
+      </c>
+      <c r="C19" s="82">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="20" spans="2:5" ht="15" x14ac:dyDescent="0.3">
+      <c r="B20" s="85" t="s">
+        <v>633</v>
+      </c>
+      <c r="C20" s="86">
+        <v>86</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
+  <tableParts count="2">
     <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
used Vlookup and Index
</commit_message>
<xml_diff>
--- a/Excel+LAB+4+Dataset_Dmart_Cleaning_Structuring.xlsx
+++ b/Excel+LAB+4+Dataset_Dmart_Cleaning_Structuring.xlsx
@@ -8,20 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Desktop\Advanced Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70C2F3D8-DE93-4D57-800C-0DA52BC76701}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{459D3787-9CC3-4FF5-8A93-B7EB38F93D24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dmart_sales_dataset" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId2"/>
     <sheet name="Sheet4" sheetId="4" r:id="rId3"/>
     <sheet name="Sheet5" sheetId="5" r:id="rId4"/>
-    <sheet name="Sheet2" sheetId="6" r:id="rId5"/>
-    <sheet name="Sheet1" sheetId="7" r:id="rId6"/>
+    <sheet name="Sheet6" sheetId="8" r:id="rId5"/>
+    <sheet name="Sheet2" sheetId="6" r:id="rId6"/>
+    <sheet name="Sheet1" sheetId="7" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Sheet1!$C$3:$C$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Sheet1!$C$3:$C$11</definedName>
     <definedName name="Category">Dmart_sales_data[Category]</definedName>
     <definedName name="city">Dmart_sales_data[Updated_City]</definedName>
     <definedName name="customer_type">Dmart_sales_data[customer_type]</definedName>
@@ -48,7 +49,7 @@
       </xcalcf:calcFeatures>
     </ext>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId7" roundtripDataChecksum="gT5L9Uh5Mkce+NjaHPxVAbIJlDW9RbqkjfO6mNdsl18="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId8" roundtripDataChecksum="gT5L9Uh5Mkce+NjaHPxVAbIJlDW9RbqkjfO6mNdsl18="/>
     </ext>
   </extLst>
 </workbook>
@@ -77,7 +78,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4671" uniqueCount="679">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4690" uniqueCount="685">
   <si>
     <t>Column1</t>
   </si>
@@ -2114,6 +2115,24 @@
   </si>
   <si>
     <t>Total Sales (subtotal)</t>
+  </si>
+  <si>
+    <t>EmpID</t>
+  </si>
+  <si>
+    <t>EmployeeID</t>
+  </si>
+  <si>
+    <t>VLOOKUP</t>
+  </si>
+  <si>
+    <t>Match of Mangesh</t>
+  </si>
+  <si>
+    <t>Using Index-Match</t>
+  </si>
+  <si>
+    <t>Using Vlookup</t>
   </si>
 </sst>
 </file>
@@ -2130,6 +2149,13 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -2285,20 +2311,13 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="12.3"/>
       <color rgb="FF333333"/>
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="20">
+  <fills count="17">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2353,11 +2372,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="5" tint="0.79998168889431442"/>
         <bgColor indexed="65"/>
       </patternFill>
@@ -2370,24 +2384,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="7" tint="0.79998168889431442"/>
         <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
       </patternFill>
     </fill>
     <fill>
@@ -2408,8 +2406,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor theme="9" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="35">
+  <borders count="42">
     <border>
       <left/>
       <right/>
@@ -2801,130 +2805,219 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="12">
+  <cellStyleXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="29" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="29" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="140">
+  <cellXfs count="150">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="9" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="9" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2945,28 +3038,28 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -2975,118 +3068,273 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="24" fillId="10" borderId="30" xfId="4" applyBorder="1"/>
-    <xf numFmtId="0" fontId="24" fillId="10" borderId="21" xfId="4" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="22" xfId="7" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="23" xfId="7" applyBorder="1"/>
-    <xf numFmtId="0" fontId="24" fillId="14" borderId="22" xfId="8" applyBorder="1"/>
-    <xf numFmtId="0" fontId="24" fillId="14" borderId="23" xfId="8" applyBorder="1"/>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="24" xfId="10" applyBorder="1"/>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="25" xfId="10" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="22" xfId="5" applyBorder="1"/>
-    <xf numFmtId="166" fontId="1" fillId="11" borderId="23" xfId="5" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="24" xfId="5" applyBorder="1"/>
-    <xf numFmtId="166" fontId="1" fillId="11" borderId="25" xfId="5" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="23" xfId="5" applyBorder="1"/>
-    <xf numFmtId="166" fontId="1" fillId="11" borderId="25" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="22" xfId="4" applyBorder="1"/>
+    <xf numFmtId="166" fontId="2" fillId="10" borderId="23" xfId="4" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="24" xfId="4" applyBorder="1"/>
+    <xf numFmtId="166" fontId="2" fillId="10" borderId="25" xfId="4" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="23" xfId="4" applyBorder="1"/>
+    <xf numFmtId="166" fontId="2" fillId="10" borderId="25" xfId="4" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="24" xfId="5" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="24" xfId="4" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="25" xfId="5" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="27" xfId="5" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="28" xfId="5" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="18" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="18" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="30" xfId="9" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="21" xfId="9" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="22" xfId="9" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="23" xfId="9" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="24" xfId="9" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="25" xfId="9" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="27" xfId="6" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="28" xfId="6" applyBorder="1"/>
-    <xf numFmtId="2" fontId="1" fillId="11" borderId="28" xfId="5" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="26" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="25" xfId="4" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="27" xfId="4" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="28" xfId="4" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="30" xfId="6" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="21" xfId="6" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="22" xfId="6" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="23" xfId="6" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="24" xfId="6" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="25" xfId="6" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="27" xfId="5" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="28" xfId="5" applyBorder="1"/>
+    <xf numFmtId="2" fontId="2" fillId="10" borderId="28" xfId="4" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="26" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="26" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="26" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="27" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="28" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="27" xfId="11" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="33" xfId="11" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="28" xfId="11" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="22" xfId="11" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="0" xfId="11" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="23" xfId="11" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="24" xfId="11" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="31" xfId="11" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="25" xfId="11" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="27" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="28" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="27" xfId="7" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="33" xfId="7" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="28" xfId="7" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="22" xfId="7" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="0" xfId="7" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="23" xfId="7" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="24" xfId="7" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="31" xfId="7" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="25" xfId="7" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="6" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="30" xfId="7" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="21" xfId="7" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="12" xfId="4" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="16" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="36" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="37" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="38" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="36" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="12">
-    <cellStyle name="20% - Accent2" xfId="5" builtinId="34"/>
-    <cellStyle name="20% - Accent3" xfId="6" builtinId="38"/>
-    <cellStyle name="20% - Accent4" xfId="9" builtinId="42"/>
-    <cellStyle name="20% - Accent5" xfId="11" builtinId="46"/>
-    <cellStyle name="60% - Accent3" xfId="7" builtinId="40"/>
-    <cellStyle name="Accent2" xfId="4" builtinId="33"/>
-    <cellStyle name="Accent4" xfId="8" builtinId="41"/>
-    <cellStyle name="Accent5" xfId="10" builtinId="45"/>
+  <cellStyles count="8">
+    <cellStyle name="20% - Accent2" xfId="4" builtinId="34"/>
+    <cellStyle name="20% - Accent3" xfId="5" builtinId="38"/>
+    <cellStyle name="20% - Accent4" xfId="6" builtinId="42"/>
+    <cellStyle name="20% - Accent5" xfId="7" builtinId="46"/>
     <cellStyle name="Good" xfId="2" builtinId="26"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Note" xfId="3" builtinId="10"/>
   </cellStyles>
-  <dxfs count="58">
+  <dxfs count="64">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -4317,28 +4565,28 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D1E78581-CDEC-49EE-B8DC-A227C0757631}" name="Dmart_sales_data" displayName="Dmart_sales_data" ref="A1:Q499" totalsRowShown="0" headerRowDxfId="57" dataDxfId="56" tableBorderDxfId="55">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D1E78581-CDEC-49EE-B8DC-A227C0757631}" name="Dmart_sales_data" displayName="Dmart_sales_data" ref="A1:Q499" totalsRowShown="0" headerRowDxfId="63" dataDxfId="62" tableBorderDxfId="61">
   <autoFilter ref="A1:Q499" xr:uid="{D1E78581-CDEC-49EE-B8DC-A227C0757631}"/>
   <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{8B304A60-B8C9-4979-B67B-B25A9B864B72}" name="Column1" dataDxfId="54"/>
-    <tableColumn id="2" xr3:uid="{2D3F64D4-436B-4836-A733-3255B375685E}" name="Region" dataDxfId="53"/>
-    <tableColumn id="15" xr3:uid="{8F8F9EC8-B524-4266-87C9-B369FF884963}" name="Updated region" dataDxfId="52"/>
-    <tableColumn id="3" xr3:uid="{E344FBA1-63F8-453C-BAB0-8696D5C5ADFA}" name="Category" dataDxfId="51"/>
-    <tableColumn id="4" xr3:uid="{EEDFF6A6-A6B8-4584-81CC-3FEFDA60E218}" name="sales" dataDxfId="50"/>
-    <tableColumn id="17" xr3:uid="{0FE78A95-ABA3-4420-9862-389F567677F4}" name="Sales_Range" dataDxfId="49">
+    <tableColumn id="1" xr3:uid="{8B304A60-B8C9-4979-B67B-B25A9B864B72}" name="Column1" dataDxfId="60"/>
+    <tableColumn id="2" xr3:uid="{2D3F64D4-436B-4836-A733-3255B375685E}" name="Region" dataDxfId="59"/>
+    <tableColumn id="15" xr3:uid="{8F8F9EC8-B524-4266-87C9-B369FF884963}" name="Updated region" dataDxfId="58"/>
+    <tableColumn id="3" xr3:uid="{E344FBA1-63F8-453C-BAB0-8696D5C5ADFA}" name="Category" dataDxfId="57"/>
+    <tableColumn id="4" xr3:uid="{EEDFF6A6-A6B8-4584-81CC-3FEFDA60E218}" name="sales" dataDxfId="56"/>
+    <tableColumn id="17" xr3:uid="{0FE78A95-ABA3-4420-9862-389F567677F4}" name="Sales_Range" dataDxfId="55">
       <calculatedColumnFormula>IF(Dmart_sales_data[[#This Row],[sales]]&gt;3000,"High Sales",IF(Dmart_sales_data[[#This Row],[sales]]&gt;1000,"Medium Sales","Low Sales"))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{B480F4CD-1259-4AB9-84E7-ADE183D66042}" name="discount" dataDxfId="48"/>
-    <tableColumn id="6" xr3:uid="{031D638C-25E8-4D1B-BC09-4AA98712CA5F}" name="quantity" dataDxfId="47"/>
-    <tableColumn id="7" xr3:uid="{6F6EB0D8-424B-4AC8-81C9-7C00315E2B39}" name="order_date" dataDxfId="46"/>
-    <tableColumn id="8" xr3:uid="{0655DCF6-A9AE-4DBC-8BCD-0DDB91A76E3F}" name="delivery_date" dataDxfId="45"/>
-    <tableColumn id="9" xr3:uid="{4A08809E-03F7-4D5D-91CC-E0D9BC4E6CCD}" name="customer_type" dataDxfId="44"/>
-    <tableColumn id="10" xr3:uid="{1B22ACAF-6F45-4EF9-BD4D-3882847DEADD}" name="customer_type2" dataDxfId="43"/>
-    <tableColumn id="11" xr3:uid="{1AAA8999-D7A1-4DB5-B4DA-131DA9CFBC1D}" name="payment_mode" dataDxfId="42"/>
-    <tableColumn id="12" xr3:uid="{47AC25B1-7621-493D-B41B-C4A660573B07}" name="profit" dataDxfId="41"/>
-    <tableColumn id="14" xr3:uid="{285DAA76-019F-4DAE-9C58-731537A4E5A8}" name="Updated_City" dataDxfId="40"/>
-    <tableColumn id="13" xr3:uid="{B1583274-EA92-4587-97FE-7E9FCE51D726}" name="city" dataDxfId="39"/>
-    <tableColumn id="18" xr3:uid="{740C088C-8609-4AAD-81B8-DF0D9B02079A}" name="Discount or Not" dataDxfId="38">
+    <tableColumn id="5" xr3:uid="{B480F4CD-1259-4AB9-84E7-ADE183D66042}" name="discount" dataDxfId="54"/>
+    <tableColumn id="6" xr3:uid="{031D638C-25E8-4D1B-BC09-4AA98712CA5F}" name="quantity" dataDxfId="53"/>
+    <tableColumn id="7" xr3:uid="{6F6EB0D8-424B-4AC8-81C9-7C00315E2B39}" name="order_date" dataDxfId="52"/>
+    <tableColumn id="8" xr3:uid="{0655DCF6-A9AE-4DBC-8BCD-0DDB91A76E3F}" name="delivery_date" dataDxfId="51"/>
+    <tableColumn id="9" xr3:uid="{4A08809E-03F7-4D5D-91CC-E0D9BC4E6CCD}" name="customer_type" dataDxfId="50"/>
+    <tableColumn id="10" xr3:uid="{1B22ACAF-6F45-4EF9-BD4D-3882847DEADD}" name="customer_type2" dataDxfId="49"/>
+    <tableColumn id="11" xr3:uid="{1AAA8999-D7A1-4DB5-B4DA-131DA9CFBC1D}" name="payment_mode" dataDxfId="48"/>
+    <tableColumn id="12" xr3:uid="{47AC25B1-7621-493D-B41B-C4A660573B07}" name="profit" dataDxfId="47"/>
+    <tableColumn id="14" xr3:uid="{285DAA76-019F-4DAE-9C58-731537A4E5A8}" name="Updated_City" dataDxfId="46"/>
+    <tableColumn id="13" xr3:uid="{B1583274-EA92-4587-97FE-7E9FCE51D726}" name="city" dataDxfId="45"/>
+    <tableColumn id="18" xr3:uid="{740C088C-8609-4AAD-81B8-DF0D9B02079A}" name="Discount or Not" dataDxfId="44">
       <calculatedColumnFormula>IF(AND(Dmart_sales_data[[#This Row],[customer_type2]]="Member",OR(Dmart_sales_data[[#This Row],[payment_mode]]="UPI",Dmart_sales_data[[#This Row],[payment_mode]]="Card")),"yes","No")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4347,7 +4595,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{0A6E07FC-F19B-467B-A96D-152F49BC9C39}" name="Table3" displayName="Table3" ref="A1:G5" totalsRowShown="0" headerRowDxfId="37" tableBorderDxfId="36">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{0A6E07FC-F19B-467B-A96D-152F49BC9C39}" name="Table3" displayName="Table3" ref="A1:G5" totalsRowShown="0" headerRowDxfId="43" tableBorderDxfId="42">
   <autoFilter ref="A1:G5" xr:uid="{0A6E07FC-F19B-467B-A96D-152F49BC9C39}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{C83CD628-8037-4113-B34D-19B4409139C8}" name="First_Name"/>
@@ -4363,7 +4611,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{591FFA04-0D55-47FF-B03F-46AEB7B93CCC}" name="Table1" displayName="Table1" ref="E7:M11" totalsRowShown="0" headerRowDxfId="35" headerRowBorderDxfId="34" tableBorderDxfId="33" totalsRowBorderDxfId="32">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{591FFA04-0D55-47FF-B03F-46AEB7B93CCC}" name="Table1" displayName="Table1" ref="E7:M11" totalsRowShown="0" headerRowDxfId="41" headerRowBorderDxfId="40" tableBorderDxfId="39" totalsRowBorderDxfId="38">
   <autoFilter ref="E7:M11" xr:uid="{591FFA04-0D55-47FF-B03F-46AEB7B93CCC}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{7A511605-F386-44F8-8EA9-21F82B34DE6B}" name="First_Name"/>
@@ -4381,24 +4629,24 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{C4582CC2-34E1-4108-B90B-B0A79AC476DF}" name="Table4" displayName="Table4" ref="H18:J23" totalsRowShown="0" headerRowBorderDxfId="31" tableBorderDxfId="30" totalsRowBorderDxfId="29">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{C4582CC2-34E1-4108-B90B-B0A79AC476DF}" name="Table4" displayName="Table4" ref="H18:J23" totalsRowShown="0" headerRowBorderDxfId="37" tableBorderDxfId="36" totalsRowBorderDxfId="35">
   <autoFilter ref="H18:J23" xr:uid="{C4582CC2-34E1-4108-B90B-B0A79AC476DF}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{2E1B0446-2B2E-4C3D-A1EE-391AF9212486}" name="Name " dataDxfId="28"/>
-    <tableColumn id="2" xr3:uid="{19AB838D-F57F-4448-AE00-5E4AA9FB304C}" name="Salary" dataDxfId="27"/>
-    <tableColumn id="3" xr3:uid="{B096BCFB-275E-45AA-A72E-D0C36078B65E}" name="Bonus" dataDxfId="26"/>
+    <tableColumn id="1" xr3:uid="{2E1B0446-2B2E-4C3D-A1EE-391AF9212486}" name="Name " dataDxfId="34"/>
+    <tableColumn id="2" xr3:uid="{19AB838D-F57F-4448-AE00-5E4AA9FB304C}" name="Salary" dataDxfId="33"/>
+    <tableColumn id="3" xr3:uid="{B096BCFB-275E-45AA-A72E-D0C36078B65E}" name="Bonus" dataDxfId="32"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{EDE8ED26-A613-4F4E-A465-CC70B9528A2A}" name="Table5" displayName="Table5" ref="H8:J13" totalsRowShown="0" headerRowDxfId="25" headerRowBorderDxfId="24" tableBorderDxfId="23" totalsRowBorderDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{EDE8ED26-A613-4F4E-A465-CC70B9528A2A}" name="Table5" displayName="Table5" ref="H8:J13" totalsRowShown="0" headerRowDxfId="31" headerRowBorderDxfId="30" tableBorderDxfId="29" totalsRowBorderDxfId="28">
   <autoFilter ref="H8:J13" xr:uid="{EDE8ED26-A613-4F4E-A465-CC70B9528A2A}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{CFB5A7CD-331C-4C43-96A8-0EF34910777D}" name="Name " dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{CB401229-AA4D-4F02-997A-EECEC42124A1}" name="Marks" dataDxfId="20"/>
-    <tableColumn id="3" xr3:uid="{032BA486-4C96-46E4-9FCC-835E6841B1B4}" name="Grade" dataDxfId="19">
+    <tableColumn id="1" xr3:uid="{CFB5A7CD-331C-4C43-96A8-0EF34910777D}" name="Name " dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{CB401229-AA4D-4F02-997A-EECEC42124A1}" name="Marks" dataDxfId="26"/>
+    <tableColumn id="3" xr3:uid="{032BA486-4C96-46E4-9FCC-835E6841B1B4}" name="Grade" dataDxfId="25">
       <calculatedColumnFormula>IF(I9&gt;=90,"A++",IF(I9&gt;75,"A+",IF(I9&gt;60,"A",IF(I9&gt;40,"B","Fail"))))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4407,12 +4655,12 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{1A0C1234-3244-41FE-AADF-1A185E3361D9}" name="Table6" displayName="Table6" ref="P17:R22" totalsRowShown="0" headerRowDxfId="18" headerRowBorderDxfId="17" tableBorderDxfId="16" totalsRowBorderDxfId="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{1A0C1234-3244-41FE-AADF-1A185E3361D9}" name="Table6" displayName="Table6" ref="P17:R22" totalsRowShown="0" headerRowDxfId="24" headerRowBorderDxfId="23" tableBorderDxfId="22" totalsRowBorderDxfId="21">
   <autoFilter ref="P17:R22" xr:uid="{1A0C1234-3244-41FE-AADF-1A185E3361D9}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{B127EBF8-5637-44F7-83D3-381997DBE027}" name="Number 1" dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{C43106B6-1733-443D-94FA-BECDAC1C755A}" name="Number 2" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{F76B590F-EE8E-45BA-9CE4-30BC585483D7}" name="Division" dataDxfId="12">
+    <tableColumn id="1" xr3:uid="{B127EBF8-5637-44F7-83D3-381997DBE027}" name="Number 1" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{C43106B6-1733-443D-94FA-BECDAC1C755A}" name="Number 2" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{F76B590F-EE8E-45BA-9CE4-30BC585483D7}" name="Division" dataDxfId="18">
       <calculatedColumnFormula>IFERROR(P18/Q18,"Cannot Devide by Zero")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4421,23 +4669,35 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{DACE1BBE-C5AD-43B2-961F-3CA9A2EB2A9F}" name="Table8" displayName="Table8" ref="B3:D9" totalsRowShown="0" headerRowBorderDxfId="11" tableBorderDxfId="10" totalsRowBorderDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{A7502A47-E98A-463F-8AA7-4D9B850FF6A3}" name="Table411" displayName="Table411" ref="D4:F9" totalsRowShown="0" headerRowBorderDxfId="4" tableBorderDxfId="5" totalsRowBorderDxfId="3">
+  <autoFilter ref="D4:F9" xr:uid="{A7502A47-E98A-463F-8AA7-4D9B850FF6A3}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{FD8EB1ED-A4EA-4B25-85B7-992ACBFDE285}" name="Name " dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{E6AC4D50-CDA2-45FD-B74D-AEEA0460D944}" name="Salary" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{138E2406-FACD-4389-AB04-04C7B4CAAAD0}" name="Bonus" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{DACE1BBE-C5AD-43B2-961F-3CA9A2EB2A9F}" name="Table8" displayName="Table8" ref="B3:D9" totalsRowShown="0" headerRowBorderDxfId="17" tableBorderDxfId="16" totalsRowBorderDxfId="15">
   <autoFilter ref="B3:D9" xr:uid="{DACE1BBE-C5AD-43B2-961F-3CA9A2EB2A9F}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{01EE2967-652D-4F72-8D82-47940A310F22}" name="Category" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{83D94CD6-8657-4942-BDBA-E7199934938C}" name="Food" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{84FFB931-E43C-401F-A346-99CA6CFFFDBA}" name="Sales" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{01EE2967-652D-4F72-8D82-47940A310F22}" name="Category" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{83D94CD6-8657-4942-BDBA-E7199934938C}" name="Food" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{84FFB931-E43C-401F-A346-99CA6CFFFDBA}" name="Sales" dataDxfId="12"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight18" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
-<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{D282ED5D-22A6-415A-A10A-2B4A8091F761}" name="Table7" displayName="Table7" ref="B16:C20" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3" totalsRowBorderDxfId="2">
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{D282ED5D-22A6-415A-A10A-2B4A8091F761}" name="Table7" displayName="Table7" ref="B16:C20" totalsRowShown="0" headerRowDxfId="11" headerRowBorderDxfId="10" tableBorderDxfId="9" totalsRowBorderDxfId="8">
   <autoFilter ref="B16:C20" xr:uid="{D282ED5D-22A6-415A-A10A-2B4A8091F761}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{0063F624-5548-4FC5-A9F7-B87EB616BE8D}" name="Data" dataDxfId="1"/>
-    <tableColumn id="2" xr3:uid="{ACA1AE24-A257-4956-B7F8-372ACF52726B}" name="Data2" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{0063F624-5548-4FC5-A9F7-B87EB616BE8D}" name="Data" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{ACA1AE24-A257-4956-B7F8-372ACF52726B}" name="Data2" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4986,12 +5246,12 @@
         <v>yes</v>
       </c>
       <c r="R5" s="1"/>
-      <c r="S5" s="119" t="s">
+      <c r="S5" s="110" t="s">
         <v>629</v>
       </c>
       <c r="T5" s="86"/>
       <c r="U5" s="1"/>
-      <c r="V5" s="108" t="s">
+      <c r="V5" s="99" t="s">
         <v>658</v>
       </c>
       <c r="W5" s="1"/>
@@ -5056,18 +5316,18 @@
         <v>No</v>
       </c>
       <c r="R6" s="1"/>
-      <c r="S6" s="98" t="s">
+      <c r="S6" s="89" t="s">
         <v>613</v>
       </c>
-      <c r="T6" s="99">
+      <c r="T6" s="90">
         <f>SUMIF(Dmart_sales_data[payment_mode],"=UPI",Dmart_sales_data[sales])</f>
         <v>386412.25</v>
       </c>
       <c r="U6" s="1"/>
-      <c r="V6" s="90" t="s">
+      <c r="V6" s="130" t="s">
         <v>650</v>
       </c>
-      <c r="W6" s="91" cm="1">
+      <c r="W6" s="131" cm="1">
         <f t="array" ref="W6">SUMIF(Region,"=North",sales)</f>
         <v>334964.16000000003</v>
       </c>
@@ -5132,13 +5392,13 @@
         <v>yes</v>
       </c>
       <c r="R7" s="1"/>
-      <c r="S7" s="98"/>
-      <c r="T7" s="99"/>
+      <c r="S7" s="89"/>
+      <c r="T7" s="90"/>
       <c r="U7" s="1"/>
-      <c r="V7" s="92" t="s">
+      <c r="V7" s="120" t="s">
         <v>651</v>
       </c>
-      <c r="W7" s="93" cm="1">
+      <c r="W7" s="122" cm="1">
         <f t="array" ref="W7">SUMIF(Region,"=South",sales)</f>
         <v>303623.68999999994</v>
       </c>
@@ -5203,18 +5463,18 @@
         <v>No</v>
       </c>
       <c r="R8" s="1"/>
-      <c r="S8" s="98" t="s">
+      <c r="S8" s="89" t="s">
         <v>614</v>
       </c>
-      <c r="T8" s="99">
+      <c r="T8" s="90">
         <f>SUMIF(Dmart_sales_data[payment_mode],"=Cash",Dmart_sales_data[sales])</f>
         <v>522964.3</v>
       </c>
       <c r="U8" s="1"/>
-      <c r="V8" s="94" t="s">
+      <c r="V8" s="120" t="s">
         <v>652</v>
       </c>
-      <c r="W8" s="95" cm="1">
+      <c r="W8" s="122" cm="1">
         <f t="array" ref="W8">SUMIF(Region,"=East",sales)</f>
         <v>337881.26999999996</v>
       </c>
@@ -5279,13 +5539,13 @@
         <v>No</v>
       </c>
       <c r="R9" s="1"/>
-      <c r="S9" s="98"/>
-      <c r="T9" s="99"/>
+      <c r="S9" s="89"/>
+      <c r="T9" s="90"/>
       <c r="U9" s="1"/>
-      <c r="V9" s="96" t="s">
+      <c r="V9" s="123" t="s">
         <v>653</v>
       </c>
-      <c r="W9" s="97" cm="1">
+      <c r="W9" s="125" cm="1">
         <f t="array" ref="W9">SUMIF(Region,"=West",sales)</f>
         <v>346200.06999999983</v>
       </c>
@@ -5350,10 +5610,10 @@
         <v>No</v>
       </c>
       <c r="R10" s="1"/>
-      <c r="S10" s="100" t="s">
+      <c r="S10" s="91" t="s">
         <v>615</v>
       </c>
-      <c r="T10" s="101">
+      <c r="T10" s="92">
         <f>SUMIF(Dmart_sales_data[payment_mode],"=Card",Dmart_sales_data[sales])</f>
         <v>413292.63999999996</v>
       </c>
@@ -5487,12 +5747,12 @@
         <v>No</v>
       </c>
       <c r="R12" s="1"/>
-      <c r="S12" s="119" t="s">
+      <c r="S12" s="110" t="s">
         <v>630</v>
       </c>
       <c r="T12" s="86"/>
       <c r="U12" s="1"/>
-      <c r="V12" s="109" t="s">
+      <c r="V12" s="100" t="s">
         <v>659</v>
       </c>
       <c r="W12" s="1"/>
@@ -5557,18 +5817,18 @@
         <v>No</v>
       </c>
       <c r="R13" s="1"/>
-      <c r="S13" s="98" t="s">
+      <c r="S13" s="89" t="s">
         <v>628</v>
       </c>
-      <c r="T13" s="99">
+      <c r="T13" s="90">
         <f>SUMIFS(Dmart_sales_data[sales],Dmart_sales_data[Category],"=Clothing",Dmart_sales_data[Updated region],"=East")</f>
         <v>60655.859999999993</v>
       </c>
       <c r="U13" s="1"/>
-      <c r="V13" s="110" t="s">
+      <c r="V13" s="101" t="s">
         <v>654</v>
       </c>
-      <c r="W13" s="111" cm="1">
+      <c r="W13" s="102" cm="1">
         <f t="array" ref="W13">COUNTIF(Region,"North")</f>
         <v>124</v>
       </c>
@@ -5633,13 +5893,13 @@
         <v>No</v>
       </c>
       <c r="R14" s="1"/>
-      <c r="S14" s="98"/>
-      <c r="T14" s="102"/>
+      <c r="S14" s="89"/>
+      <c r="T14" s="93"/>
       <c r="U14" s="1"/>
-      <c r="V14" s="112" t="s">
+      <c r="V14" s="103" t="s">
         <v>655</v>
       </c>
-      <c r="W14" s="113" cm="1">
+      <c r="W14" s="104" cm="1">
         <f t="array" ref="W14">COUNTIF(Region,"North")</f>
         <v>124</v>
       </c>
@@ -5704,18 +5964,18 @@
         <v>No</v>
       </c>
       <c r="R15" s="1"/>
-      <c r="S15" s="100" t="s">
+      <c r="S15" s="91" t="s">
         <v>631</v>
       </c>
-      <c r="T15" s="103">
+      <c r="T15" s="94">
         <f>SUMIFS(Dmart_sales_data[sales],Dmart_sales_data[Category],"Electronics",Dmart_sales_data[Updated region],"North",Dmart_sales_data[discount],"&gt;0.40")</f>
         <v>36091.269999999997</v>
       </c>
       <c r="U15" s="19"/>
-      <c r="V15" s="112" t="s">
+      <c r="V15" s="103" t="s">
         <v>656</v>
       </c>
-      <c r="W15" s="113" cm="1">
+      <c r="W15" s="104" cm="1">
         <f t="array" ref="W15">COUNTIF(Region,"East")</f>
         <v>125</v>
       </c>
@@ -5783,10 +6043,10 @@
       <c r="S16" s="1"/>
       <c r="T16" s="19"/>
       <c r="U16" s="19"/>
-      <c r="V16" s="114" t="s">
+      <c r="V16" s="105" t="s">
         <v>657</v>
       </c>
-      <c r="W16" s="115" cm="1">
+      <c r="W16" s="106" cm="1">
         <f t="array" ref="W16">COUNTIF(Region,"West")</f>
         <v>125</v>
       </c>
@@ -5917,7 +6177,7 @@
         <v>yes</v>
       </c>
       <c r="R18" s="1"/>
-      <c r="S18" s="120" t="s">
+      <c r="S18" s="111" t="s">
         <v>638</v>
       </c>
       <c r="T18" s="88"/>
@@ -5985,18 +6245,18 @@
         <v>No</v>
       </c>
       <c r="R19" s="1"/>
-      <c r="S19" s="104" t="s">
+      <c r="S19" s="95" t="s">
         <v>637</v>
       </c>
-      <c r="T19" s="105">
+      <c r="T19" s="96">
         <f>COUNT(sales)</f>
         <v>498</v>
       </c>
       <c r="U19" s="1"/>
-      <c r="V19" s="116" t="s">
+      <c r="V19" s="107" t="s">
         <v>660</v>
       </c>
-      <c r="W19" s="117" cm="1">
+      <c r="W19" s="108" cm="1">
         <f t="array" ref="W19">SUMIF(order_date,"&lt;1-01-2024",sales)</f>
         <v>654586.69000000018</v>
       </c>
@@ -6064,10 +6324,10 @@
       <c r="S20" s="1"/>
       <c r="T20" s="1"/>
       <c r="U20" s="1"/>
-      <c r="V20" s="106" t="s">
+      <c r="V20" s="97" t="s">
         <v>661</v>
       </c>
-      <c r="W20" s="118" cm="1">
+      <c r="W20" s="109" cm="1">
         <f t="array" ref="W20">SUMIF(order_date,"&gt;30-06-2024",sales)</f>
         <v>368049.34999999992</v>
       </c>
@@ -6200,18 +6460,18 @@
         <v>No</v>
       </c>
       <c r="R22" s="1"/>
-      <c r="S22" s="98" t="s">
+      <c r="S22" s="89" t="s">
         <v>640</v>
       </c>
-      <c r="T22" s="102" cm="1">
+      <c r="T22" s="93" cm="1">
         <f t="array" ref="T22">COUNTIF(transactions,"Cash")</f>
         <v>185</v>
       </c>
       <c r="U22" s="1"/>
-      <c r="V22" s="106" t="s">
+      <c r="V22" s="97" t="s">
         <v>662</v>
       </c>
-      <c r="W22" s="107" cm="1">
+      <c r="W22" s="98" cm="1">
         <f t="array" ref="W22">COUNTIF(payment_mode,"UPI")</f>
         <v>149</v>
       </c>
@@ -6276,10 +6536,10 @@
         <v>No</v>
       </c>
       <c r="R23" s="1"/>
-      <c r="S23" s="98" t="s">
+      <c r="S23" s="89" t="s">
         <v>641</v>
       </c>
-      <c r="T23" s="102" cm="1">
+      <c r="T23" s="93" cm="1">
         <f t="array" ref="T23">COUNTIF(transactions,"Card")</f>
         <v>164</v>
       </c>
@@ -6346,18 +6606,18 @@
         <v>No</v>
       </c>
       <c r="R24" s="1"/>
-      <c r="S24" s="100" t="s">
+      <c r="S24" s="91" t="s">
         <v>642</v>
       </c>
-      <c r="T24" s="105" cm="1">
+      <c r="T24" s="96" cm="1">
         <f t="array" ref="T24">COUNTIF(transactions,"UPI")</f>
         <v>149</v>
       </c>
       <c r="U24" s="1"/>
-      <c r="V24" s="89" t="s">
+      <c r="V24" s="132" t="s">
         <v>612</v>
       </c>
-      <c r="W24" s="1">
+      <c r="W24" s="132">
         <f>SUM(sales)</f>
         <v>1322669.1900000023</v>
       </c>
@@ -6422,18 +6682,18 @@
         <v>No</v>
       </c>
       <c r="R25" s="1"/>
-      <c r="S25" s="106" t="s">
+      <c r="S25" s="97" t="s">
         <v>643</v>
       </c>
-      <c r="T25" s="107" cm="1">
+      <c r="T25" s="98" cm="1">
         <f t="array" ref="T25">COUNTIF(sales,"&gt;4000")</f>
         <v>115</v>
       </c>
       <c r="U25" s="1"/>
-      <c r="V25" s="139" t="s">
+      <c r="V25" s="132" t="s">
         <v>678</v>
       </c>
-      <c r="W25" s="1" cm="1">
+      <c r="W25" s="132" cm="1">
         <f t="array" ref="W25">SUBTOTAL(9,sales)</f>
         <v>1322669.1900000023</v>
       </c>
@@ -6694,7 +6954,7 @@
         <v>No</v>
       </c>
       <c r="R29" s="1"/>
-      <c r="S29" s="119" t="s">
+      <c r="S29" s="110" t="s">
         <v>648</v>
       </c>
       <c r="T29" s="86"/>
@@ -6762,10 +7022,10 @@
         <v>yes</v>
       </c>
       <c r="R30" s="1"/>
-      <c r="S30" s="98" t="s">
+      <c r="S30" s="89" t="s">
         <v>644</v>
       </c>
-      <c r="T30" s="102" cm="1">
+      <c r="T30" s="93" cm="1">
         <f t="array" ref="T30">COUNTIFS(sales,"&gt;4000",Region,"North")</f>
         <v>32</v>
       </c>
@@ -6833,10 +7093,10 @@
         <v>No</v>
       </c>
       <c r="R31" s="1"/>
-      <c r="S31" s="98" t="s">
+      <c r="S31" s="89" t="s">
         <v>645</v>
       </c>
-      <c r="T31" s="102" cm="1">
+      <c r="T31" s="93" cm="1">
         <f t="array" ref="T31">COUNTIFS(sales,"&gt;4000",Region,"East")</f>
         <v>29</v>
       </c>
@@ -6904,10 +7164,10 @@
         <v>No</v>
       </c>
       <c r="R32" s="1"/>
-      <c r="S32" s="98" t="s">
+      <c r="S32" s="89" t="s">
         <v>646</v>
       </c>
-      <c r="T32" s="102" cm="1">
+      <c r="T32" s="93" cm="1">
         <f t="array" ref="T32">COUNTIFS(sales,"&gt;4000",Region,"South")</f>
         <v>27</v>
       </c>
@@ -6975,10 +7235,10 @@
         <v>No</v>
       </c>
       <c r="R33" s="1"/>
-      <c r="S33" s="100" t="s">
+      <c r="S33" s="91" t="s">
         <v>647</v>
       </c>
-      <c r="T33" s="105" cm="1">
+      <c r="T33" s="96" cm="1">
         <f t="array" ref="T33">COUNTIFS(sales,"&gt;4000",Region,"West")</f>
         <v>27</v>
       </c>
@@ -7178,10 +7438,10 @@
         <v>No</v>
       </c>
       <c r="R36" s="1"/>
-      <c r="S36" s="121" t="s">
+      <c r="S36" s="112" t="s">
         <v>649</v>
       </c>
-      <c r="T36" s="122" cm="1">
+      <c r="T36" s="113" cm="1">
         <f t="array" ref="T36">COUNTIFS(customer_type,"Member",payment_mode,"Card") + COUNTIFS(customer_type,"Member",payment_mode,"UPI")</f>
         <v>97</v>
       </c>
@@ -51781,7 +52041,7 @@
       <c r="Z1000" s="1"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="6" type="noConversion"/>
+  <phoneticPr fontId="7" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
   <tableParts count="1">
@@ -52394,64 +52654,64 @@
     </row>
     <row r="28" spans="8:18" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="29" spans="8:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="H29" s="126" t="s">
+      <c r="H29" s="117" t="s">
         <v>673</v>
       </c>
-      <c r="I29" s="127" t="s">
+      <c r="I29" s="118" t="s">
         <v>663</v>
       </c>
-      <c r="J29" s="128" t="s">
+      <c r="J29" s="119" t="s">
         <v>664</v>
       </c>
     </row>
     <row r="30" spans="8:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="H30" s="129" t="s">
+      <c r="H30" s="120" t="s">
         <v>665</v>
       </c>
-      <c r="I30" s="130" t="s">
+      <c r="I30" s="121" t="s">
         <v>668</v>
       </c>
-      <c r="J30" s="131">
+      <c r="J30" s="122">
         <v>1001</v>
       </c>
-      <c r="L30" s="124" t="s">
+      <c r="L30" s="115" t="s">
         <v>672</v>
       </c>
-      <c r="M30" s="125">
+      <c r="M30" s="116">
         <f>COUNTIF(J30:J33,1001)</f>
         <v>2</v>
       </c>
     </row>
     <row r="31" spans="8:18" x14ac:dyDescent="0.3">
-      <c r="H31" s="129" t="s">
+      <c r="H31" s="120" t="s">
         <v>617</v>
       </c>
-      <c r="I31" s="130" t="s">
+      <c r="I31" s="121" t="s">
         <v>669</v>
       </c>
-      <c r="J31" s="131">
+      <c r="J31" s="122">
         <v>1002</v>
       </c>
     </row>
     <row r="32" spans="8:18" x14ac:dyDescent="0.3">
-      <c r="H32" s="129" t="s">
+      <c r="H32" s="120" t="s">
         <v>666</v>
       </c>
-      <c r="I32" s="130" t="s">
+      <c r="I32" s="121" t="s">
         <v>670</v>
       </c>
-      <c r="J32" s="131">
+      <c r="J32" s="122">
         <v>1001</v>
       </c>
     </row>
     <row r="33" spans="8:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="H33" s="132" t="s">
+      <c r="H33" s="123" t="s">
         <v>667</v>
       </c>
-      <c r="I33" s="133" t="s">
+      <c r="I33" s="124" t="s">
         <v>671</v>
       </c>
-      <c r="J33" s="134">
+      <c r="J33" s="125">
         <v>1002</v>
       </c>
     </row>
@@ -52466,6 +52726,187 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA220B27-A011-45EC-B903-F7F36FAFED8F}">
+  <dimension ref="C2:J14"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="4" max="4" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="15.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="C2" s="30" t="s">
+        <v>681</v>
+      </c>
+    </row>
+    <row r="4" spans="3:10" ht="18" x14ac:dyDescent="0.35">
+      <c r="C4" s="138" t="s">
+        <v>679</v>
+      </c>
+      <c r="D4" s="44" t="s">
+        <v>584</v>
+      </c>
+      <c r="E4" s="45" t="s">
+        <v>602</v>
+      </c>
+      <c r="F4" s="46" t="s">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="5" spans="3:10" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C5" s="139">
+        <v>1001</v>
+      </c>
+      <c r="D5" s="42" t="s">
+        <v>585</v>
+      </c>
+      <c r="E5" s="41">
+        <v>70000</v>
+      </c>
+      <c r="F5" s="43">
+        <f>IF(E5&gt;$L$19,(E5*15%),IF(E5&gt;$L$20,(E5*10%),IF(E5&gt;$L$21,(E5*5%))))</f>
+        <v>10500</v>
+      </c>
+    </row>
+    <row r="6" spans="3:10" ht="18" x14ac:dyDescent="0.3">
+      <c r="C6" s="38">
+        <v>1002</v>
+      </c>
+      <c r="D6" s="42" t="s">
+        <v>586</v>
+      </c>
+      <c r="E6" s="41">
+        <v>50000</v>
+      </c>
+      <c r="F6" s="43">
+        <f>IF(E6&gt;$L$19,(E6*15%),IF(E6&gt;$L$20,(E6*10%),IF(E6&gt;$L$21,(E6*5%),"No Bonus")))</f>
+        <v>7500</v>
+      </c>
+      <c r="H6" s="143" t="s">
+        <v>684</v>
+      </c>
+      <c r="I6" s="133"/>
+      <c r="J6" s="134"/>
+    </row>
+    <row r="7" spans="3:10" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C7" s="139">
+        <v>1003</v>
+      </c>
+      <c r="D7" s="42" t="s">
+        <v>587</v>
+      </c>
+      <c r="E7" s="41">
+        <v>45000</v>
+      </c>
+      <c r="F7" s="43">
+        <f>IF(E7&gt;$L$19,(E7*15%),IF(E7&gt;$L$20,(E7*10%),IF(E7&gt;$L$21,(E7*5%),"No Bonus")))</f>
+        <v>6750</v>
+      </c>
+      <c r="H7" s="144" t="s">
+        <v>680</v>
+      </c>
+      <c r="I7" s="140" t="s">
+        <v>603</v>
+      </c>
+      <c r="J7" s="145" t="s">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="8" spans="3:10" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C8" s="38">
+        <v>1004</v>
+      </c>
+      <c r="D8" s="42" t="s">
+        <v>588</v>
+      </c>
+      <c r="E8" s="41">
+        <v>75000</v>
+      </c>
+      <c r="F8" s="43">
+        <f>IF(E8&gt;$L$19,(E8*15%),IF(E8&gt;$L$20,(E8*10%),IF(E8&gt;$L$21,(E8*5%))))</f>
+        <v>11250</v>
+      </c>
+      <c r="H8" s="141">
+        <v>1003</v>
+      </c>
+      <c r="I8" s="142">
+        <f>VLOOKUP(H8,C5:F9,MATCH(Table411[[#Headers],[Bonus]],C4:F4,0),FALSE)</f>
+        <v>6750</v>
+      </c>
+      <c r="J8" s="142">
+        <f>VLOOKUP(H8,C5:F9,MATCH(E8,C8:F8,0),FALSE)</f>
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="9" spans="3:10" ht="18" x14ac:dyDescent="0.3">
+      <c r="C9" s="139">
+        <v>1005</v>
+      </c>
+      <c r="D9" s="47" t="s">
+        <v>599</v>
+      </c>
+      <c r="E9" s="48">
+        <v>55000</v>
+      </c>
+      <c r="F9" s="49">
+        <f>IF(E9&gt;$L$19,(E9*15%),IF(E9&gt;$L$20,(E9*10%),IF(E9&gt;$L$21,(E9*5%))))</f>
+        <v>8250</v>
+      </c>
+    </row>
+    <row r="10" spans="3:10" x14ac:dyDescent="0.3">
+      <c r="H10" t="s">
+        <v>682</v>
+      </c>
+      <c r="I10">
+        <f>MATCH(D8,Table411[[Name ]],0)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D12" s="146" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="13" spans="3:10" ht="18" x14ac:dyDescent="0.35">
+      <c r="D13" s="147" t="s">
+        <v>679</v>
+      </c>
+      <c r="E13" s="148" t="s">
+        <v>602</v>
+      </c>
+      <c r="F13" s="149" t="s">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="14" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D14" s="135">
+        <v>1002</v>
+      </c>
+      <c r="E14" s="136">
+        <f>INDEX(C5:F9,MATCH(D14,C4:C9,0),MATCH(Table411[[#Headers],[Salary]],C4:F4,0))</f>
+        <v>45000</v>
+      </c>
+      <c r="F14" s="137">
+        <f>INDEX(C5:F9,MATCH(D14,C4:C9,0),MATCH(Table411[[#Headers],[Bonus]],C4:F4,0))</f>
+        <v>6750</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H8 D14" xr:uid="{7FE34A3E-67F7-4932-98C3-CC8B2FC31DD4}">
+      <formula1>$C$5:$C$9</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEF34D78-29E1-4CCD-BF36-EC79D09F917E}">
   <dimension ref="B3:G20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -52616,7 +53057,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3FD06C3-E835-4820-937A-C092995027EB}">
   <dimension ref="C2:J11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -52628,25 +53069,25 @@
   <sheetData>
     <row r="2" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="3" spans="3:10" ht="21" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C3" s="136" t="s">
+      <c r="C3" s="127" t="s">
         <v>632</v>
       </c>
-      <c r="D3" s="137"/>
-      <c r="E3" s="137"/>
+      <c r="D3" s="128"/>
+      <c r="E3" s="128"/>
     </row>
     <row r="4" spans="3:10" ht="15" x14ac:dyDescent="0.3">
-      <c r="C4" s="138">
+      <c r="C4" s="129">
         <v>120</v>
       </c>
-      <c r="D4" s="138"/>
-      <c r="E4" s="138"/>
+      <c r="D4" s="129"/>
+      <c r="E4" s="129"/>
     </row>
     <row r="5" spans="3:10" ht="15" x14ac:dyDescent="0.3">
-      <c r="C5" s="138">
+      <c r="C5" s="129">
         <v>10</v>
       </c>
-      <c r="D5" s="138"/>
-      <c r="E5" s="138"/>
+      <c r="D5" s="129"/>
+      <c r="E5" s="129"/>
       <c r="F5" s="30" t="s">
         <v>675</v>
       </c>
@@ -52663,11 +53104,11 @@
       </c>
     </row>
     <row r="6" spans="3:10" ht="15" hidden="1" x14ac:dyDescent="0.3">
-      <c r="C6" s="138">
+      <c r="C6" s="129">
         <v>150</v>
       </c>
-      <c r="D6" s="138"/>
-      <c r="E6" s="138"/>
+      <c r="D6" s="129"/>
+      <c r="E6" s="129"/>
       <c r="F6" s="30" t="s">
         <v>674</v>
       </c>
@@ -52677,32 +53118,32 @@
       </c>
     </row>
     <row r="7" spans="3:10" ht="15" hidden="1" x14ac:dyDescent="0.3">
-      <c r="C7" s="138">
+      <c r="C7" s="129">
         <v>23</v>
       </c>
-      <c r="D7" s="135"/>
-      <c r="E7" s="135"/>
+      <c r="D7" s="126"/>
+      <c r="E7" s="126"/>
     </row>
     <row r="8" spans="3:10" ht="15" x14ac:dyDescent="0.3">
-      <c r="C8" s="138">
+      <c r="C8" s="129">
         <v>65</v>
       </c>
     </row>
     <row r="9" spans="3:10" ht="15" x14ac:dyDescent="0.3">
-      <c r="C9" s="138">
+      <c r="C9" s="129">
         <v>55</v>
       </c>
-      <c r="H9" s="123" t="s">
+      <c r="H9" s="114" t="s">
         <v>677</v>
       </c>
     </row>
     <row r="10" spans="3:10" ht="15" x14ac:dyDescent="0.3">
-      <c r="C10" s="138">
+      <c r="C10" s="129">
         <v>56</v>
       </c>
     </row>
     <row r="11" spans="3:10" ht="15" x14ac:dyDescent="0.3">
-      <c r="C11" s="138">
+      <c r="C11" s="129">
         <v>58</v>
       </c>
     </row>

</xml_diff>

<commit_message>
learnt Vloolup and Hlookup
</commit_message>
<xml_diff>
--- a/Excel+LAB+4+Dataset_Dmart_Cleaning_Structuring.xlsx
+++ b/Excel+LAB+4+Dataset_Dmart_Cleaning_Structuring.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Desktop\Advanced Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1F12615-E19C-4E8D-B918-3F9939495E35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C8AD002-37FD-46B9-9707-4B0693FAE04A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dmart_sales_dataset" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="Sheet6" sheetId="8" r:id="rId5"/>
     <sheet name="Sheet2" sheetId="6" r:id="rId6"/>
     <sheet name="Sheet1" sheetId="7" r:id="rId7"/>
+    <sheet name="Hlookup" sheetId="9" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Sheet1!$C$3:$C$11</definedName>
@@ -49,14 +50,14 @@
       </xcalcf:calcFeatures>
     </ext>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId8" roundtripDataChecksum="gT5L9Uh5Mkce+NjaHPxVAbIJlDW9RbqkjfO6mNdsl18="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId9" roundtripDataChecksum="gT5L9Uh5Mkce+NjaHPxVAbIJlDW9RbqkjfO6mNdsl18="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -78,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4692" uniqueCount="686">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4707" uniqueCount="696">
   <si>
     <t>Column1</t>
   </si>
@@ -2126,9 +2127,6 @@
     <t>VLOOKUP</t>
   </si>
   <si>
-    <t>Match of Mangesh</t>
-  </si>
-  <si>
     <t>Using Index-Match</t>
   </si>
   <si>
@@ -2136,6 +2134,39 @@
   </si>
   <si>
     <t xml:space="preserve">Employee Id </t>
+  </si>
+  <si>
+    <t>Jan</t>
+  </si>
+  <si>
+    <t>Feb</t>
+  </si>
+  <si>
+    <t>Mar</t>
+  </si>
+  <si>
+    <t>Apr</t>
+  </si>
+  <si>
+    <t>May</t>
+  </si>
+  <si>
+    <t>Cost</t>
+  </si>
+  <si>
+    <t>Travel</t>
+  </si>
+  <si>
+    <t>Profit</t>
+  </si>
+  <si>
+    <t>Month</t>
+  </si>
+  <si>
+    <t>Using Hlookup and Match</t>
+  </si>
+  <si>
+    <t xml:space="preserve">May </t>
   </si>
 </sst>
 </file>
@@ -2147,11 +2178,18 @@
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="&quot;₹&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="28" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -2319,8 +2357,14 @@
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="17">
+  <fills count="18">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2415,8 +2459,14 @@
         <bgColor theme="9" tint="0.79998168889431442"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="42">
+  <borders count="47">
     <border>
       <left/>
       <right/>
@@ -2901,126 +2951,198 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="8">
+  <cellStyleXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="24" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="23" fillId="9" borderId="29" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="24" fillId="9" borderId="29" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="154">
+  <cellXfs count="165">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="9" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="9" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="9" xfId="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
@@ -3041,28 +3163,28 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -3071,144 +3193,162 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="22" xfId="4" applyBorder="1"/>
-    <xf numFmtId="166" fontId="2" fillId="10" borderId="23" xfId="4" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="24" xfId="4" applyBorder="1"/>
-    <xf numFmtId="166" fontId="2" fillId="10" borderId="25" xfId="4" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="23" xfId="4" applyBorder="1"/>
-    <xf numFmtId="166" fontId="2" fillId="10" borderId="25" xfId="4" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="22" xfId="4" applyBorder="1"/>
+    <xf numFmtId="166" fontId="3" fillId="10" borderId="23" xfId="4" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="24" xfId="4" applyBorder="1"/>
+    <xf numFmtId="166" fontId="3" fillId="10" borderId="25" xfId="4" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="23" xfId="4" applyBorder="1"/>
+    <xf numFmtId="166" fontId="3" fillId="10" borderId="25" xfId="4" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="24" xfId="4" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="24" xfId="4" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="25" xfId="4" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="27" xfId="4" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="28" xfId="4" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="14" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="14" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="30" xfId="6" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="21" xfId="6" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="22" xfId="6" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="23" xfId="6" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="24" xfId="6" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="25" xfId="6" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="27" xfId="5" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="28" xfId="5" applyBorder="1"/>
-    <xf numFmtId="2" fontId="2" fillId="10" borderId="28" xfId="4" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="26" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="25" xfId="4" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="27" xfId="4" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="28" xfId="4" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="30" xfId="6" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="21" xfId="6" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="22" xfId="6" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="23" xfId="6" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="24" xfId="6" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="25" xfId="6" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="27" xfId="5" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="28" xfId="5" applyBorder="1"/>
+    <xf numFmtId="2" fontId="3" fillId="10" borderId="28" xfId="4" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="26" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="26" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="26" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="8" borderId="27" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="24" fillId="8" borderId="28" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="27" xfId="7" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="33" xfId="7" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="28" xfId="7" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="22" xfId="7" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="0" xfId="7" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="23" xfId="7" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="24" xfId="7" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="31" xfId="7" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="25" xfId="7" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="27" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="28" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="27" xfId="7" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="33" xfId="7" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="28" xfId="7" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="22" xfId="7" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="7" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="23" xfId="7" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="24" xfId="7" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="31" xfId="7" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="25" xfId="7" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="21" fillId="6" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="6" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="6" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="30" xfId="7" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="21" xfId="7" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="12" xfId="4" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="30" xfId="7" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="21" xfId="7" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="12" xfId="4" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="16" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="36" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="36" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="14" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="37" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="37" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="38" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="38" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="36" xfId="3" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="36" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="29" xfId="3" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="29" xfId="3" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="39" xfId="7" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="41" xfId="7" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="44" xfId="7" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="42" xfId="7" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="45" xfId="7" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="43" xfId="7" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="46" xfId="7" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="12" xfId="8" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="17" borderId="12" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="8">
+  <cellStyles count="9">
     <cellStyle name="20% - Accent2" xfId="4" builtinId="34"/>
     <cellStyle name="20% - Accent3" xfId="5" builtinId="38"/>
     <cellStyle name="20% - Accent4" xfId="6" builtinId="42"/>
     <cellStyle name="20% - Accent5" xfId="7" builtinId="46"/>
+    <cellStyle name="20% - Accent6" xfId="8" builtinId="50"/>
     <cellStyle name="Good" xfId="2" builtinId="26"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3395,137 +3535,6 @@
       </border>
     </dxf>
     <dxf>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="14"/>
-        <color theme="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left/>
         <right style="thin">
@@ -4562,6 +4571,137 @@
       </fill>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -4576,28 +4716,28 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D1E78581-CDEC-49EE-B8DC-A227C0757631}" name="Dmart_sales_data" displayName="Dmart_sales_data" ref="A1:Q499" totalsRowShown="0" headerRowDxfId="63" dataDxfId="62" tableBorderDxfId="61">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D1E78581-CDEC-49EE-B8DC-A227C0757631}" name="Dmart_sales_data" displayName="Dmart_sales_data" ref="A1:Q499" totalsRowShown="0" headerRowDxfId="57" dataDxfId="56" tableBorderDxfId="55">
   <autoFilter ref="A1:Q499" xr:uid="{D1E78581-CDEC-49EE-B8DC-A227C0757631}"/>
   <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{8B304A60-B8C9-4979-B67B-B25A9B864B72}" name="Column1" dataDxfId="60"/>
-    <tableColumn id="2" xr3:uid="{2D3F64D4-436B-4836-A733-3255B375685E}" name="Region" dataDxfId="59"/>
-    <tableColumn id="15" xr3:uid="{8F8F9EC8-B524-4266-87C9-B369FF884963}" name="Updated region" dataDxfId="58"/>
-    <tableColumn id="3" xr3:uid="{E344FBA1-63F8-453C-BAB0-8696D5C5ADFA}" name="Category" dataDxfId="57"/>
-    <tableColumn id="4" xr3:uid="{EEDFF6A6-A6B8-4584-81CC-3FEFDA60E218}" name="sales" dataDxfId="56"/>
-    <tableColumn id="17" xr3:uid="{0FE78A95-ABA3-4420-9862-389F567677F4}" name="Sales_Range" dataDxfId="55">
+    <tableColumn id="1" xr3:uid="{8B304A60-B8C9-4979-B67B-B25A9B864B72}" name="Column1" dataDxfId="54"/>
+    <tableColumn id="2" xr3:uid="{2D3F64D4-436B-4836-A733-3255B375685E}" name="Region" dataDxfId="53"/>
+    <tableColumn id="15" xr3:uid="{8F8F9EC8-B524-4266-87C9-B369FF884963}" name="Updated region" dataDxfId="52"/>
+    <tableColumn id="3" xr3:uid="{E344FBA1-63F8-453C-BAB0-8696D5C5ADFA}" name="Category" dataDxfId="51"/>
+    <tableColumn id="4" xr3:uid="{EEDFF6A6-A6B8-4584-81CC-3FEFDA60E218}" name="sales" dataDxfId="50"/>
+    <tableColumn id="17" xr3:uid="{0FE78A95-ABA3-4420-9862-389F567677F4}" name="Sales_Range" dataDxfId="49">
       <calculatedColumnFormula>IF(Dmart_sales_data[[#This Row],[sales]]&gt;3000,"High Sales",IF(Dmart_sales_data[[#This Row],[sales]]&gt;1000,"Medium Sales","Low Sales"))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{B480F4CD-1259-4AB9-84E7-ADE183D66042}" name="discount" dataDxfId="54"/>
-    <tableColumn id="6" xr3:uid="{031D638C-25E8-4D1B-BC09-4AA98712CA5F}" name="quantity" dataDxfId="53"/>
-    <tableColumn id="7" xr3:uid="{6F6EB0D8-424B-4AC8-81C9-7C00315E2B39}" name="order_date" dataDxfId="52"/>
-    <tableColumn id="8" xr3:uid="{0655DCF6-A9AE-4DBC-8BCD-0DDB91A76E3F}" name="delivery_date" dataDxfId="51"/>
-    <tableColumn id="9" xr3:uid="{4A08809E-03F7-4D5D-91CC-E0D9BC4E6CCD}" name="customer_type" dataDxfId="50"/>
-    <tableColumn id="10" xr3:uid="{1B22ACAF-6F45-4EF9-BD4D-3882847DEADD}" name="customer_type2" dataDxfId="49"/>
-    <tableColumn id="11" xr3:uid="{1AAA8999-D7A1-4DB5-B4DA-131DA9CFBC1D}" name="payment_mode" dataDxfId="48"/>
-    <tableColumn id="12" xr3:uid="{47AC25B1-7621-493D-B41B-C4A660573B07}" name="profit" dataDxfId="47"/>
-    <tableColumn id="14" xr3:uid="{285DAA76-019F-4DAE-9C58-731537A4E5A8}" name="Updated_City" dataDxfId="46"/>
-    <tableColumn id="13" xr3:uid="{B1583274-EA92-4587-97FE-7E9FCE51D726}" name="city" dataDxfId="45"/>
-    <tableColumn id="18" xr3:uid="{740C088C-8609-4AAD-81B8-DF0D9B02079A}" name="Discount or Not" dataDxfId="44">
+    <tableColumn id="5" xr3:uid="{B480F4CD-1259-4AB9-84E7-ADE183D66042}" name="discount" dataDxfId="48"/>
+    <tableColumn id="6" xr3:uid="{031D638C-25E8-4D1B-BC09-4AA98712CA5F}" name="quantity" dataDxfId="47"/>
+    <tableColumn id="7" xr3:uid="{6F6EB0D8-424B-4AC8-81C9-7C00315E2B39}" name="order_date" dataDxfId="46"/>
+    <tableColumn id="8" xr3:uid="{0655DCF6-A9AE-4DBC-8BCD-0DDB91A76E3F}" name="delivery_date" dataDxfId="45"/>
+    <tableColumn id="9" xr3:uid="{4A08809E-03F7-4D5D-91CC-E0D9BC4E6CCD}" name="customer_type" dataDxfId="44"/>
+    <tableColumn id="10" xr3:uid="{1B22ACAF-6F45-4EF9-BD4D-3882847DEADD}" name="customer_type2" dataDxfId="43"/>
+    <tableColumn id="11" xr3:uid="{1AAA8999-D7A1-4DB5-B4DA-131DA9CFBC1D}" name="payment_mode" dataDxfId="42"/>
+    <tableColumn id="12" xr3:uid="{47AC25B1-7621-493D-B41B-C4A660573B07}" name="profit" dataDxfId="41"/>
+    <tableColumn id="14" xr3:uid="{285DAA76-019F-4DAE-9C58-731537A4E5A8}" name="Updated_City" dataDxfId="40"/>
+    <tableColumn id="13" xr3:uid="{B1583274-EA92-4587-97FE-7E9FCE51D726}" name="city" dataDxfId="39"/>
+    <tableColumn id="18" xr3:uid="{740C088C-8609-4AAD-81B8-DF0D9B02079A}" name="Discount or Not" dataDxfId="38">
       <calculatedColumnFormula>IF(AND(Dmart_sales_data[[#This Row],[customer_type2]]="Member",OR(Dmart_sales_data[[#This Row],[payment_mode]]="UPI",Dmart_sales_data[[#This Row],[payment_mode]]="Card")),"yes","No")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4606,7 +4746,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{0A6E07FC-F19B-467B-A96D-152F49BC9C39}" name="Table3" displayName="Table3" ref="A1:G5" totalsRowShown="0" headerRowDxfId="43" tableBorderDxfId="42">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{0A6E07FC-F19B-467B-A96D-152F49BC9C39}" name="Table3" displayName="Table3" ref="A1:G5" totalsRowShown="0" headerRowDxfId="37" tableBorderDxfId="36">
   <autoFilter ref="A1:G5" xr:uid="{0A6E07FC-F19B-467B-A96D-152F49BC9C39}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{C83CD628-8037-4113-B34D-19B4409139C8}" name="First_Name"/>
@@ -4622,7 +4762,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{591FFA04-0D55-47FF-B03F-46AEB7B93CCC}" name="Table1" displayName="Table1" ref="E7:M11" totalsRowShown="0" headerRowDxfId="41" headerRowBorderDxfId="40" tableBorderDxfId="39" totalsRowBorderDxfId="38">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{591FFA04-0D55-47FF-B03F-46AEB7B93CCC}" name="Table1" displayName="Table1" ref="E7:M11" totalsRowShown="0" headerRowDxfId="35" headerRowBorderDxfId="34" tableBorderDxfId="33" totalsRowBorderDxfId="32">
   <autoFilter ref="E7:M11" xr:uid="{591FFA04-0D55-47FF-B03F-46AEB7B93CCC}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{7A511605-F386-44F8-8EA9-21F82B34DE6B}" name="First_Name"/>
@@ -4640,24 +4780,24 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{C4582CC2-34E1-4108-B90B-B0A79AC476DF}" name="Table4" displayName="Table4" ref="H18:J23" totalsRowShown="0" headerRowBorderDxfId="37" tableBorderDxfId="36" totalsRowBorderDxfId="35">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{C4582CC2-34E1-4108-B90B-B0A79AC476DF}" name="Table4" displayName="Table4" ref="H18:J23" totalsRowShown="0" headerRowBorderDxfId="31" tableBorderDxfId="30" totalsRowBorderDxfId="29">
   <autoFilter ref="H18:J23" xr:uid="{C4582CC2-34E1-4108-B90B-B0A79AC476DF}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{2E1B0446-2B2E-4C3D-A1EE-391AF9212486}" name="Name " dataDxfId="34"/>
-    <tableColumn id="2" xr3:uid="{19AB838D-F57F-4448-AE00-5E4AA9FB304C}" name="Salary" dataDxfId="33"/>
-    <tableColumn id="3" xr3:uid="{B096BCFB-275E-45AA-A72E-D0C36078B65E}" name="Bonus" dataDxfId="32"/>
+    <tableColumn id="1" xr3:uid="{2E1B0446-2B2E-4C3D-A1EE-391AF9212486}" name="Name " dataDxfId="28"/>
+    <tableColumn id="2" xr3:uid="{19AB838D-F57F-4448-AE00-5E4AA9FB304C}" name="Salary" dataDxfId="27"/>
+    <tableColumn id="3" xr3:uid="{B096BCFB-275E-45AA-A72E-D0C36078B65E}" name="Bonus" dataDxfId="26"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{EDE8ED26-A613-4F4E-A465-CC70B9528A2A}" name="Table5" displayName="Table5" ref="H8:J13" totalsRowShown="0" headerRowDxfId="31" headerRowBorderDxfId="30" tableBorderDxfId="29" totalsRowBorderDxfId="28">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{EDE8ED26-A613-4F4E-A465-CC70B9528A2A}" name="Table5" displayName="Table5" ref="H8:J13" totalsRowShown="0" headerRowDxfId="25" headerRowBorderDxfId="24" tableBorderDxfId="23" totalsRowBorderDxfId="22">
   <autoFilter ref="H8:J13" xr:uid="{EDE8ED26-A613-4F4E-A465-CC70B9528A2A}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{CFB5A7CD-331C-4C43-96A8-0EF34910777D}" name="Name " dataDxfId="27"/>
-    <tableColumn id="2" xr3:uid="{CB401229-AA4D-4F02-997A-EECEC42124A1}" name="Marks" dataDxfId="26"/>
-    <tableColumn id="3" xr3:uid="{032BA486-4C96-46E4-9FCC-835E6841B1B4}" name="Grade" dataDxfId="25">
+    <tableColumn id="1" xr3:uid="{CFB5A7CD-331C-4C43-96A8-0EF34910777D}" name="Name " dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{CB401229-AA4D-4F02-997A-EECEC42124A1}" name="Marks" dataDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{032BA486-4C96-46E4-9FCC-835E6841B1B4}" name="Grade" dataDxfId="19">
       <calculatedColumnFormula>IF(I9&gt;=90,"A++",IF(I9&gt;75,"A+",IF(I9&gt;60,"A",IF(I9&gt;40,"B","Fail"))))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4666,12 +4806,12 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{1A0C1234-3244-41FE-AADF-1A185E3361D9}" name="Table6" displayName="Table6" ref="P17:R22" totalsRowShown="0" headerRowDxfId="24" headerRowBorderDxfId="23" tableBorderDxfId="22" totalsRowBorderDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{1A0C1234-3244-41FE-AADF-1A185E3361D9}" name="Table6" displayName="Table6" ref="P17:R22" totalsRowShown="0" headerRowDxfId="18" headerRowBorderDxfId="17" tableBorderDxfId="16" totalsRowBorderDxfId="15">
   <autoFilter ref="P17:R22" xr:uid="{1A0C1234-3244-41FE-AADF-1A185E3361D9}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{B127EBF8-5637-44F7-83D3-381997DBE027}" name="Number 1" dataDxfId="20"/>
-    <tableColumn id="2" xr3:uid="{C43106B6-1733-443D-94FA-BECDAC1C755A}" name="Number 2" dataDxfId="19"/>
-    <tableColumn id="3" xr3:uid="{F76B590F-EE8E-45BA-9CE4-30BC585483D7}" name="Division" dataDxfId="18">
+    <tableColumn id="1" xr3:uid="{B127EBF8-5637-44F7-83D3-381997DBE027}" name="Number 1" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{C43106B6-1733-443D-94FA-BECDAC1C755A}" name="Number 2" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{F76B590F-EE8E-45BA-9CE4-30BC585483D7}" name="Division" dataDxfId="12">
       <calculatedColumnFormula>IFERROR(P18/Q18,"Cannot Devide by Zero")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4680,12 +4820,12 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{A7502A47-E98A-463F-8AA7-4D9B850FF6A3}" name="Table411" displayName="Table411" ref="D4:F9" totalsRowShown="0" headerRowBorderDxfId="17" tableBorderDxfId="16" totalsRowBorderDxfId="15">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{A7502A47-E98A-463F-8AA7-4D9B850FF6A3}" name="Table411" displayName="Table411" ref="D4:F9" totalsRowShown="0" headerRowBorderDxfId="63" tableBorderDxfId="62" totalsRowBorderDxfId="61">
   <autoFilter ref="D4:F9" xr:uid="{A7502A47-E98A-463F-8AA7-4D9B850FF6A3}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{FD8EB1ED-A4EA-4B25-85B7-992ACBFDE285}" name="Name " dataDxfId="14"/>
-    <tableColumn id="2" xr3:uid="{E6AC4D50-CDA2-45FD-B74D-AEEA0460D944}" name="Salary" dataDxfId="13"/>
-    <tableColumn id="3" xr3:uid="{138E2406-FACD-4389-AB04-04C7B4CAAAD0}" name="Bonus" dataDxfId="12"/>
+    <tableColumn id="1" xr3:uid="{FD8EB1ED-A4EA-4B25-85B7-992ACBFDE285}" name="Name " dataDxfId="60"/>
+    <tableColumn id="2" xr3:uid="{E6AC4D50-CDA2-45FD-B74D-AEEA0460D944}" name="Salary" dataDxfId="59"/>
+    <tableColumn id="3" xr3:uid="{138E2406-FACD-4389-AB04-04C7B4CAAAD0}" name="Bonus" dataDxfId="58"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight21" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -52052,7 +52192,7 @@
       <c r="Z1000" s="1"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="7" type="noConversion"/>
+  <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
   <tableParts count="1">
@@ -52738,7 +52878,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EA220B27-A011-45EC-B903-F7F36FAFED8F}">
-  <dimension ref="C2:J18"/>
+  <dimension ref="C2:J14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="4" max="4" width="15.77734375" bestFit="1" customWidth="1"/>
@@ -52795,8 +52935,8 @@
         <f>IF(E6&gt;$L$19,(E6*15%),IF(E6&gt;$L$20,(E6*10%),IF(E6&gt;$L$21,(E6*5%),"No Bonus")))</f>
         <v>7500</v>
       </c>
-      <c r="H6" s="143" t="s">
-        <v>684</v>
+      <c r="H6" s="153" t="s">
+        <v>683</v>
       </c>
       <c r="I6" s="133"/>
       <c r="J6" s="134"/>
@@ -52815,13 +52955,13 @@
         <f>IF(E7&gt;$L$19,(E7*15%),IF(E7&gt;$L$20,(E7*10%),IF(E7&gt;$L$21,(E7*5%),"No Bonus")))</f>
         <v>6750</v>
       </c>
-      <c r="H7" s="144" t="s">
+      <c r="H7" s="143" t="s">
         <v>680</v>
       </c>
       <c r="I7" s="140" t="s">
         <v>603</v>
       </c>
-      <c r="J7" s="145" t="s">
+      <c r="J7" s="144" t="s">
         <v>617</v>
       </c>
     </row>
@@ -52866,40 +53006,31 @@
         <v>8250</v>
       </c>
     </row>
-    <row r="10" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="H10" t="s">
+    <row r="12" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D12" s="145" t="s">
         <v>682</v>
       </c>
-      <c r="I10">
-        <f>MATCH(D8,Table411[[Name ]],0)</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="12" spans="3:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D12" s="146" t="s">
-        <v>683</v>
-      </c>
-      <c r="H12" s="152" t="s">
-        <v>685</v>
-      </c>
-      <c r="I12" s="153" t="s">
+      <c r="H12" s="151" t="s">
+        <v>684</v>
+      </c>
+      <c r="I12" s="152" t="s">
         <v>603</v>
       </c>
     </row>
     <row r="13" spans="3:10" ht="18" x14ac:dyDescent="0.35">
-      <c r="D13" s="147" t="s">
+      <c r="D13" s="146" t="s">
         <v>679</v>
       </c>
-      <c r="E13" s="148" t="s">
+      <c r="E13" s="147" t="s">
         <v>602</v>
       </c>
-      <c r="F13" s="149" t="s">
+      <c r="F13" s="148" t="s">
         <v>603</v>
       </c>
-      <c r="H13" s="150">
+      <c r="H13" s="149">
         <v>1004</v>
       </c>
-      <c r="I13" s="151">
+      <c r="I13" s="150">
         <f>VLOOKUP(H13,C5:F9,4,FALSE)</f>
         <v>11250</v>
       </c>
@@ -52915,24 +53046,6 @@
       <c r="F14" s="137">
         <f>INDEX(C5:F9,MATCH(D14,C4:C9,0),MATCH(Table411[[#Headers],[Bonus]],C4:F4,0))</f>
         <v>6750</v>
-      </c>
-    </row>
-    <row r="16" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="D16">
-        <v>1003</v>
-      </c>
-      <c r="E16">
-        <f>INDEX(C5:F9,MATCH(D16,C5:C9,0),MATCH(Table411[[#Headers],[Bonus]],C4:F4,0))</f>
-        <v>6750</v>
-      </c>
-      <c r="H16">
-        <f>MATCH(H13,C5:C9,0)</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="18" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D18">
-        <v>1005</v>
       </c>
     </row>
   </sheetData>
@@ -53194,4 +53307,171 @@
   <autoFilter ref="C3:C11" xr:uid="{F3FD06C3-E835-4820-937A-C092995027EB}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18A97367-C201-4A03-88AF-E85974923122}">
+  <dimension ref="D5:I15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="5" max="5" width="21.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="5" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="D5" s="163"/>
+      <c r="E5" s="164" t="s">
+        <v>685</v>
+      </c>
+      <c r="F5" s="164" t="s">
+        <v>686</v>
+      </c>
+      <c r="G5" s="164" t="s">
+        <v>687</v>
+      </c>
+      <c r="H5" s="164" t="s">
+        <v>688</v>
+      </c>
+      <c r="I5" s="164" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="6" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="D6" s="164" t="s">
+        <v>690</v>
+      </c>
+      <c r="E6" s="163">
+        <v>100</v>
+      </c>
+      <c r="F6" s="163">
+        <v>585</v>
+      </c>
+      <c r="G6" s="163">
+        <v>333</v>
+      </c>
+      <c r="H6" s="163">
+        <v>562</v>
+      </c>
+      <c r="I6" s="163">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="7" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="D7" s="164" t="s">
+        <v>691</v>
+      </c>
+      <c r="E7" s="163">
+        <v>100.5</v>
+      </c>
+      <c r="F7" s="163">
+        <v>563</v>
+      </c>
+      <c r="G7" s="163">
+        <v>555</v>
+      </c>
+      <c r="H7" s="163">
+        <v>234</v>
+      </c>
+      <c r="I7" s="163">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="8" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="D8" s="164" t="s">
+        <v>617</v>
+      </c>
+      <c r="E8" s="163">
+        <v>2000</v>
+      </c>
+      <c r="F8" s="163">
+        <v>5000</v>
+      </c>
+      <c r="G8" s="163">
+        <v>6000</v>
+      </c>
+      <c r="H8" s="163">
+        <v>4000</v>
+      </c>
+      <c r="I8" s="163">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="9" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="D9" s="164" t="s">
+        <v>692</v>
+      </c>
+      <c r="E9" s="163">
+        <v>400</v>
+      </c>
+      <c r="F9" s="163">
+        <v>500</v>
+      </c>
+      <c r="G9" s="163">
+        <v>300</v>
+      </c>
+      <c r="H9" s="163">
+        <v>300</v>
+      </c>
+      <c r="I9" s="163">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="11" spans="4:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E11" s="155" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="12" spans="4:9" x14ac:dyDescent="0.3">
+      <c r="E12" s="156" t="s">
+        <v>693</v>
+      </c>
+      <c r="F12" s="157" t="s">
+        <v>687</v>
+      </c>
+      <c r="G12" s="154" t="s">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="13" spans="4:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E13" s="158" t="s">
+        <v>617</v>
+      </c>
+      <c r="F13" s="159">
+        <f>HLOOKUP($G$5,$D$5:$I$9,MATCH(E13,$D$5:$D$9,0),FALSE)</f>
+        <v>6000</v>
+      </c>
+      <c r="G13">
+        <f>VLOOKUP(D8,D6:I10,MATCH($I$5,$D$5:$I$5,0),FALSE)</f>
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="14" spans="4:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E14" s="160" t="s">
+        <v>691</v>
+      </c>
+      <c r="F14" s="161">
+        <f>HLOOKUP($G$5,$D$5:$I$9,MATCH(E14,$D$5:$D$9,0),FALSE)</f>
+        <v>555</v>
+      </c>
+      <c r="G14">
+        <f t="shared" ref="G14:G15" si="0">VLOOKUP(D9,D7:I11,MATCH($I$5,$D$5:$I$5,0),FALSE)</f>
+        <v>200</v>
+      </c>
+    </row>
+    <row r="15" spans="4:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E15" s="162" t="s">
+        <v>692</v>
+      </c>
+      <c r="F15" s="161">
+        <f>HLOOKUP($G$5,$D$5:$I$9,MATCH(E15,$D$5:$D$9,0),FALSE)</f>
+        <v>300</v>
+      </c>
+      <c r="G15" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="27" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>